<commit_message>
Softer age marks, poster tint, per-film title fonts, simpler rating dialog
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q8auJtZCZpXRhnY2W8Jqqg
</commit_message>
<xml_diff>
--- a/data/films.xlsx
+++ b/data/films.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -452,9 +452,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -505,10 +503,15 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>8. 영문폰트: 상세 페이지 영문 제목 글꼴. classic·elegant·noir·epic·typewriter·mono·bold·scifi·gothic·western·retro·script·hand·comic·light·neon 중 하나 (비우면 classic).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11"/>
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>수정 후: python tools/xlsx_to_json.py 를 실행하면 data/films.json 이 갱신됩니다.</t>
         </is>
@@ -525,7 +528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U51"/>
+  <dimension ref="A1:V51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -549,6 +552,7 @@
     <col width="9" customWidth="1" min="19" max="19"/>
     <col width="26" customWidth="1" min="20" max="20"/>
     <col width="8" customWidth="1" min="21" max="21"/>
+    <col width="11" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -657,6 +661,11 @@
           <t>문양</t>
         </is>
       </c>
+      <c r="V1" s="5" t="inlineStr">
+        <is>
+          <t>영문폰트</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -754,6 +763,11 @@
           <t>split</t>
         </is>
       </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>elegant</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -851,6 +865,11 @@
           <t>rings</t>
         </is>
       </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>noir</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -948,6 +967,11 @@
           <t>peaks</t>
         </is>
       </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>western</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -1045,6 +1069,11 @@
           <t>grid</t>
         </is>
       </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>typewriter</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -1140,6 +1169,11 @@
       <c r="U6" s="3" t="inlineStr">
         <is>
           <t>arch</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>epic</t>
         </is>
       </c>
     </row>
@@ -1235,6 +1269,11 @@
           <t>rays</t>
         </is>
       </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>bold</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -1328,6 +1367,11 @@
           <t>dots</t>
         </is>
       </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>script</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -1421,6 +1465,11 @@
           <t>sun</t>
         </is>
       </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>bold</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -1514,6 +1563,11 @@
           <t>grid</t>
         </is>
       </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>mono</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -1607,6 +1661,11 @@
           <t>bands</t>
         </is>
       </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>typewriter</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -1704,6 +1763,11 @@
           <t>waves</t>
         </is>
       </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>elegant</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -1801,6 +1865,11 @@
           <t>bands</t>
         </is>
       </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>epic</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -1896,6 +1965,11 @@
       <c r="U14" s="3" t="inlineStr">
         <is>
           <t>peaks</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>bold</t>
         </is>
       </c>
     </row>
@@ -1991,6 +2065,11 @@
           <t>dots</t>
         </is>
       </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>hand</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -2084,6 +2163,11 @@
           <t>split</t>
         </is>
       </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>bold</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -2177,6 +2261,11 @@
           <t>grid</t>
         </is>
       </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>typewriter</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -2270,6 +2359,11 @@
           <t>trees</t>
         </is>
       </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>gothic</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -2363,6 +2457,11 @@
           <t>split</t>
         </is>
       </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>elegant</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -2456,6 +2555,11 @@
           <t>trees</t>
         </is>
       </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>retro</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -2549,6 +2653,11 @@
           <t>peaks</t>
         </is>
       </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>classic</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -2644,6 +2753,11 @@
       <c r="U22" s="3" t="inlineStr">
         <is>
           <t>rays</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>gothic</t>
         </is>
       </c>
     </row>
@@ -2739,6 +2853,11 @@
           <t>sun</t>
         </is>
       </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>bold</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -2832,6 +2951,11 @@
           <t>rings</t>
         </is>
       </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>scifi</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -2925,6 +3049,11 @@
           <t>bands</t>
         </is>
       </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>western</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -3018,6 +3147,11 @@
           <t>rays</t>
         </is>
       </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>bold</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -3111,6 +3245,11 @@
           <t>rings</t>
         </is>
       </c>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>scifi</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
@@ -3204,6 +3343,11 @@
           <t>rings</t>
         </is>
       </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>noir</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -3297,6 +3441,11 @@
           <t>arch</t>
         </is>
       </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>light</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
@@ -3390,6 +3539,11 @@
           <t>waves</t>
         </is>
       </c>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>noir</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -3483,6 +3637,11 @@
           <t>grid</t>
         </is>
       </c>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>classic</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
@@ -3576,6 +3735,11 @@
           <t>arch</t>
         </is>
       </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>hand</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
@@ -3669,6 +3833,11 @@
           <t>trees</t>
         </is>
       </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>epic</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
@@ -3766,6 +3935,11 @@
           <t>rings</t>
         </is>
       </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>script</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -3861,6 +4035,11 @@
       <c r="U35" s="3" t="inlineStr">
         <is>
           <t>dots</t>
+        </is>
+      </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>hand</t>
         </is>
       </c>
     </row>
@@ -3956,6 +4135,11 @@
           <t>dots</t>
         </is>
       </c>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>comic</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
@@ -4049,6 +4233,11 @@
           <t>arch</t>
         </is>
       </c>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>script</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
@@ -4142,6 +4331,11 @@
           <t>dots</t>
         </is>
       </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>hand</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
@@ -4235,6 +4429,11 @@
           <t>grid</t>
         </is>
       </c>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>scifi</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
@@ -4328,6 +4527,11 @@
           <t>rays</t>
         </is>
       </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>light</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
@@ -4421,6 +4625,11 @@
           <t>dots</t>
         </is>
       </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>retro</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
@@ -4514,6 +4723,11 @@
           <t>rays</t>
         </is>
       </c>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>noir</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
@@ -4607,6 +4821,11 @@
           <t>rays</t>
         </is>
       </c>
+      <c r="V43" t="inlineStr">
+        <is>
+          <t>typewriter</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
@@ -4700,6 +4919,11 @@
           <t>rays</t>
         </is>
       </c>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>script</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
@@ -4793,6 +5017,11 @@
           <t>sun</t>
         </is>
       </c>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>elegant</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
@@ -4886,6 +5115,11 @@
           <t>bands</t>
         </is>
       </c>
+      <c r="V46" t="inlineStr">
+        <is>
+          <t>retro</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
@@ -4979,6 +5213,11 @@
           <t>trees</t>
         </is>
       </c>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>light</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
@@ -5072,6 +5311,11 @@
           <t>arch</t>
         </is>
       </c>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>bold</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
@@ -5165,6 +5409,11 @@
           <t>bands</t>
         </is>
       </c>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>neon</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
@@ -5258,6 +5507,11 @@
           <t>arch</t>
         </is>
       </c>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>script</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
@@ -5351,9 +5605,14 @@
           <t>split</t>
         </is>
       </c>
+      <c r="V51" t="inlineStr">
+        <is>
+          <t>retro</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <dataValidations count="3">
+  <dataValidations count="4">
     <dataValidation sqref="S2:S500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"전체,12,15,18"</formula1>
     </dataValidation>
@@ -5362,6 +5621,9 @@
     </dataValidation>
     <dataValidation sqref="U2:U500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"sun,waves,bands,rings,split,peaks,arch,rays,grid,dots,trees"</formula1>
+    </dataValidation>
+    <dataValidation sqref="V2:V500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"classic,elegant,noir,epic,typewriter,mono,bold,scifi,gothic,western,retro,script,hand,comic,light,neon"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Full-width film page, mood accent fonts, background colour override
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q8auJtZCZpXRhnY2W8Jqqg
</commit_message>
<xml_diff>
--- a/data/films.xlsx
+++ b/data/films.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -452,7 +452,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -509,9 +508,16 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>9. 배경색: 상세 페이지 배경 색을 직접 정할 때만 #aabbcc 형식으로. 비우면 포스터의 대표색을 어둡게 낮춰 씁니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>수정 후: python tools/xlsx_to_json.py 를 실행하면 data/films.json 이 갱신됩니다.</t>
         </is>
@@ -528,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V51"/>
+  <dimension ref="A1:W51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -553,6 +559,7 @@
     <col width="26" customWidth="1" min="20" max="20"/>
     <col width="8" customWidth="1" min="21" max="21"/>
     <col width="11" customWidth="1" min="22" max="22"/>
+    <col width="11" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -666,6 +673,11 @@
           <t>영문폰트</t>
         </is>
       </c>
+      <c r="W1" s="5" t="inlineStr">
+        <is>
+          <t>배경색</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -1566,6 +1578,11 @@
       <c r="V10" t="inlineStr">
         <is>
           <t>mono</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>#1f3a6b</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Build TMDB data in a GitHub Action, spreadsheet colours, transfer link, README
- tools/xlsx_to_json.py fetches posters, Korean ratings and streaming
  services at build time, verifies TMDB IDs and writes a report
- GitHub Action runs it on spreadsheet changes and weekly; TMDB key is
  a repo secret, no longer in the page
- Film page colours come from the spreadsheet for all 50 films
- Smaller age marks, two-line intros, favicon and share preview
- Move ratings to another device with a link; back button always home

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q8auJtZCZpXRhnY2W8Jqqg
</commit_message>
<xml_diff>
--- a/data/films.xlsx
+++ b/data/films.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,8 +35,11 @@
       <b val="1"/>
       <sz val="14"/>
     </font>
+    <font>
+      <color rgb="00F1E8D6"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="53">
     <fill>
       <patternFill/>
     </fill>
@@ -46,6 +49,256 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="004E0F1D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002b2116"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001d1c19"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002a2017"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001d2333"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002c1215"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00241a0a"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001c1a35"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002a140a"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001a2b4f"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001c2226"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001c1c1c"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001e1f17"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001a2229"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0010241a"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001c2230"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001b1f1c"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000f2020"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002a1f17"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00142219"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001c2228"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002a1012"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002e160b"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00142030"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002a2015"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000f151d"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0015161c"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001d1714"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001d2224"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001a2024"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002a1612"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0013253a"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0012221a"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002a1b10"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0013203a"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002a1030"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0022143a"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0017204a"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002b2010"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001a1e45"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0013283a"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0018120d"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00142231"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002c1512"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002a2016"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0026162f"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0024190f"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001e1d16"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000f2522"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00222020"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002b1210"/>
       </patternFill>
     </fill>
   </fills>
@@ -61,7 +314,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -74,6 +327,56 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="18" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="20" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="21" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="22" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="23" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="24" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="25" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="26" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="27" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="28" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="29" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="30" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="31" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="32" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="33" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="34" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="35" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="36" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="37" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="38" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="39" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="40" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="41" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="42" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="43" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="44" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="45" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="46" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="47" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="48" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="49" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="50" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="51" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="52" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -452,6 +755,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -511,7 +815,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>9. 배경색: 상세 페이지 배경 색을 직접 정할 때만 #aabbcc 형식으로. 비우면 포스터의 대표색을 어둡게 낮춰 씁니다.</t>
+          <t>9. 배경색: 상세 페이지 전체 배경색(#aabbcc). 셀 색이 실제 색입니다. 밝은 글씨가 잘 보이도록 어두운 색을 쓰세요.</t>
         </is>
       </c>
     </row>
@@ -519,7 +823,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>수정 후: python tools/xlsx_to_json.py 를 실행하면 data/films.json 이 갱신됩니다.</t>
+          <t>수정 후: GitHub 저장소의 data/films.xlsx 를 이 파일로 교체해 올리면, 자동으로 data/films.json 이 만들어지고 사이트에 반영됩니다(1~3분).</t>
         </is>
       </c>
     </row>
@@ -780,6 +1084,11 @@
           <t>elegant</t>
         </is>
       </c>
+      <c r="W2" s="6" t="inlineStr">
+        <is>
+          <t>#2b2116</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -882,6 +1191,11 @@
           <t>noir</t>
         </is>
       </c>
+      <c r="W3" s="7" t="inlineStr">
+        <is>
+          <t>#1d1c19</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -984,6 +1298,11 @@
           <t>western</t>
         </is>
       </c>
+      <c r="W4" s="8" t="inlineStr">
+        <is>
+          <t>#2a2017</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -1086,6 +1405,11 @@
           <t>typewriter</t>
         </is>
       </c>
+      <c r="W5" s="9" t="inlineStr">
+        <is>
+          <t>#1d2333</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -1186,6 +1510,11 @@
       <c r="V6" t="inlineStr">
         <is>
           <t>epic</t>
+        </is>
+      </c>
+      <c r="W6" s="10" t="inlineStr">
+        <is>
+          <t>#2c1215</t>
         </is>
       </c>
     </row>
@@ -1286,6 +1615,11 @@
           <t>bold</t>
         </is>
       </c>
+      <c r="W7" s="11" t="inlineStr">
+        <is>
+          <t>#241a0a</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -1384,6 +1718,11 @@
           <t>script</t>
         </is>
       </c>
+      <c r="W8" s="12" t="inlineStr">
+        <is>
+          <t>#1c1a35</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -1482,6 +1821,11 @@
           <t>bold</t>
         </is>
       </c>
+      <c r="W9" s="13" t="inlineStr">
+        <is>
+          <t>#2a140a</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -1580,9 +1924,9 @@
           <t>mono</t>
         </is>
       </c>
-      <c r="W10" t="inlineStr">
-        <is>
-          <t>#1f3a6b</t>
+      <c r="W10" s="14" t="inlineStr">
+        <is>
+          <t>#1a2b4f</t>
         </is>
       </c>
     </row>
@@ -1683,6 +2027,11 @@
           <t>typewriter</t>
         </is>
       </c>
+      <c r="W11" s="15" t="inlineStr">
+        <is>
+          <t>#1c2226</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -1785,6 +2134,11 @@
           <t>elegant</t>
         </is>
       </c>
+      <c r="W12" s="16" t="inlineStr">
+        <is>
+          <t>#1c1c1c</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -1887,6 +2241,11 @@
           <t>epic</t>
         </is>
       </c>
+      <c r="W13" s="17" t="inlineStr">
+        <is>
+          <t>#1e1f17</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -1987,6 +2346,11 @@
       <c r="V14" t="inlineStr">
         <is>
           <t>bold</t>
+        </is>
+      </c>
+      <c r="W14" s="18" t="inlineStr">
+        <is>
+          <t>#1a2229</t>
         </is>
       </c>
     </row>
@@ -2087,6 +2451,11 @@
           <t>hand</t>
         </is>
       </c>
+      <c r="W15" s="19" t="inlineStr">
+        <is>
+          <t>#10241a</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -2185,6 +2554,11 @@
           <t>bold</t>
         </is>
       </c>
+      <c r="W16" s="20" t="inlineStr">
+        <is>
+          <t>#1c2230</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -2283,6 +2657,11 @@
           <t>typewriter</t>
         </is>
       </c>
+      <c r="W17" s="21" t="inlineStr">
+        <is>
+          <t>#1b1f1c</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -2381,6 +2760,11 @@
           <t>gothic</t>
         </is>
       </c>
+      <c r="W18" s="22" t="inlineStr">
+        <is>
+          <t>#0f2020</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -2479,6 +2863,11 @@
           <t>elegant</t>
         </is>
       </c>
+      <c r="W19" s="23" t="inlineStr">
+        <is>
+          <t>#2a1f17</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -2577,6 +2966,11 @@
           <t>retro</t>
         </is>
       </c>
+      <c r="W20" s="24" t="inlineStr">
+        <is>
+          <t>#142219</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -2675,6 +3069,11 @@
           <t>classic</t>
         </is>
       </c>
+      <c r="W21" s="25" t="inlineStr">
+        <is>
+          <t>#1c2228</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -2775,6 +3174,11 @@
       <c r="V22" t="inlineStr">
         <is>
           <t>gothic</t>
+        </is>
+      </c>
+      <c r="W22" s="26" t="inlineStr">
+        <is>
+          <t>#2a1012</t>
         </is>
       </c>
     </row>
@@ -2875,6 +3279,11 @@
           <t>bold</t>
         </is>
       </c>
+      <c r="W23" s="27" t="inlineStr">
+        <is>
+          <t>#2e160b</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -2973,6 +3382,11 @@
           <t>scifi</t>
         </is>
       </c>
+      <c r="W24" s="28" t="inlineStr">
+        <is>
+          <t>#142030</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -3071,6 +3485,11 @@
           <t>western</t>
         </is>
       </c>
+      <c r="W25" s="29" t="inlineStr">
+        <is>
+          <t>#2a2015</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -3169,6 +3588,11 @@
           <t>bold</t>
         </is>
       </c>
+      <c r="W26" s="30" t="inlineStr">
+        <is>
+          <t>#0f151d</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -3267,6 +3691,11 @@
           <t>scifi</t>
         </is>
       </c>
+      <c r="W27" s="31" t="inlineStr">
+        <is>
+          <t>#15161c</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
@@ -3365,6 +3794,11 @@
           <t>noir</t>
         </is>
       </c>
+      <c r="W28" s="32" t="inlineStr">
+        <is>
+          <t>#1d1714</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -3463,6 +3897,11 @@
           <t>light</t>
         </is>
       </c>
+      <c r="W29" s="33" t="inlineStr">
+        <is>
+          <t>#1d2224</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
@@ -3561,6 +4000,11 @@
           <t>noir</t>
         </is>
       </c>
+      <c r="W30" s="34" t="inlineStr">
+        <is>
+          <t>#1a2024</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -3659,6 +4103,11 @@
           <t>classic</t>
         </is>
       </c>
+      <c r="W31" s="35" t="inlineStr">
+        <is>
+          <t>#2a1612</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
@@ -3757,6 +4206,11 @@
           <t>hand</t>
         </is>
       </c>
+      <c r="W32" s="36" t="inlineStr">
+        <is>
+          <t>#13253a</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
@@ -3855,6 +4309,11 @@
           <t>epic</t>
         </is>
       </c>
+      <c r="W33" s="37" t="inlineStr">
+        <is>
+          <t>#12221a</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
@@ -3957,6 +4416,11 @@
           <t>script</t>
         </is>
       </c>
+      <c r="W34" s="38" t="inlineStr">
+        <is>
+          <t>#2a1b10</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -4057,6 +4521,11 @@
       <c r="V35" t="inlineStr">
         <is>
           <t>hand</t>
+        </is>
+      </c>
+      <c r="W35" s="39" t="inlineStr">
+        <is>
+          <t>#13203a</t>
         </is>
       </c>
     </row>
@@ -4157,6 +4626,11 @@
           <t>comic</t>
         </is>
       </c>
+      <c r="W36" s="40" t="inlineStr">
+        <is>
+          <t>#2a1030</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
@@ -4255,6 +4729,11 @@
           <t>script</t>
         </is>
       </c>
+      <c r="W37" s="41" t="inlineStr">
+        <is>
+          <t>#22143a</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
@@ -4353,6 +4832,11 @@
           <t>hand</t>
         </is>
       </c>
+      <c r="W38" s="42" t="inlineStr">
+        <is>
+          <t>#17204a</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
@@ -4451,6 +4935,11 @@
           <t>scifi</t>
         </is>
       </c>
+      <c r="W39" s="43" t="inlineStr">
+        <is>
+          <t>#2b2010</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
@@ -4549,6 +5038,11 @@
           <t>light</t>
         </is>
       </c>
+      <c r="W40" s="44" t="inlineStr">
+        <is>
+          <t>#1a1e45</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
@@ -4647,6 +5141,11 @@
           <t>retro</t>
         </is>
       </c>
+      <c r="W41" s="45" t="inlineStr">
+        <is>
+          <t>#13283a</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
@@ -4745,6 +5244,11 @@
           <t>noir</t>
         </is>
       </c>
+      <c r="W42" s="46" t="inlineStr">
+        <is>
+          <t>#18120d</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
@@ -4843,6 +5347,11 @@
           <t>typewriter</t>
         </is>
       </c>
+      <c r="W43" s="47" t="inlineStr">
+        <is>
+          <t>#142231</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
@@ -4941,6 +5450,11 @@
           <t>script</t>
         </is>
       </c>
+      <c r="W44" s="48" t="inlineStr">
+        <is>
+          <t>#2c1512</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
@@ -5039,6 +5553,11 @@
           <t>elegant</t>
         </is>
       </c>
+      <c r="W45" s="49" t="inlineStr">
+        <is>
+          <t>#2a2016</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
@@ -5137,6 +5656,11 @@
           <t>retro</t>
         </is>
       </c>
+      <c r="W46" s="50" t="inlineStr">
+        <is>
+          <t>#26162f</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
@@ -5235,6 +5759,11 @@
           <t>light</t>
         </is>
       </c>
+      <c r="W47" s="51" t="inlineStr">
+        <is>
+          <t>#24190f</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
@@ -5333,6 +5862,11 @@
           <t>bold</t>
         </is>
       </c>
+      <c r="W48" s="52" t="inlineStr">
+        <is>
+          <t>#1e1d16</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
@@ -5431,6 +5965,11 @@
           <t>neon</t>
         </is>
       </c>
+      <c r="W49" s="53" t="inlineStr">
+        <is>
+          <t>#0f2522</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
@@ -5529,6 +6068,11 @@
           <t>script</t>
         </is>
       </c>
+      <c r="W50" s="54" t="inlineStr">
+        <is>
+          <t>#222020</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
@@ -5625,6 +6169,11 @@
       <c r="V51" t="inlineStr">
         <is>
           <t>retro</t>
+        </is>
+      </c>
+      <c r="W51" s="55" t="inlineStr">
+        <is>
+          <t>#2b1210</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Per-film point colour on film pages, stored in the spreadsheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q8auJtZCZpXRhnY2W8Jqqg
</commit_message>
<xml_diff>
--- a/data/films.xlsx
+++ b/data/films.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="54">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,6 +37,206 @@
     </font>
     <font>
       <color rgb="00F1E8D6"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00e2b45c"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00e7c35a"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00d9b88a"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00f2ad96"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00e3c27a"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00f0b43c"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00f3cf6a"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00f39a4b"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00acccff"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00b9c9d6"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00cfcfcf"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00d4c48e"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00a9cbe0"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00f9a491"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00e6c79a"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00b7c7a8"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00d9b468"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00eab48a"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00b8d98a"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00c7d3dc"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00f09a9a"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00ff9a4a"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="008fc3e6"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00d8b47e"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="008fb1d6"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00d8c79a"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00f0a597"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00b8c6c8"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00a8c0cf"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00e0b06a"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00f8ae9a"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00a9d08a"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00e8b878"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00f2c36b"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00ffa6d0"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00ffb347"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00ffd75a"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00f0c060"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00f5b39a"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00ffc96b"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00d4b06a"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00c9d8e8"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00f0c87a"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00ecd08a"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00ffa84a"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00e3a96a"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00b9cc8a"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00f2d45c"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00eab0b0"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00f2c94c"/>
     </font>
   </fonts>
   <fills count="53">
@@ -314,7 +514,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="106">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -377,6 +577,56 @@
     <xf numFmtId="0" fontId="3" fillId="50" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="51" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="52" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="24" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="25" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="27" fillId="26" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="27" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="28" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="29" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="31" fillId="30" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="32" fillId="31" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="33" fillId="32" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="34" fillId="33" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="35" fillId="34" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="36" fillId="35" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="37" fillId="36" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="38" fillId="37" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="39" fillId="38" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="40" fillId="39" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="41" fillId="40" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="42" fillId="41" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="43" fillId="42" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="44" fillId="43" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="45" fillId="44" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="46" fillId="45" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="47" fillId="46" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="48" fillId="47" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="49" fillId="48" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="50" fillId="49" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="51" fillId="50" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="52" fillId="51" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="53" fillId="52" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -742,7 +992,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -819,9 +1069,16 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>10. 포인트색: 상세 페이지의 영문 제목·소제목·번호·항목 이름 색(#aabbcc). 셀에 배경색 위 실제 모습이 보입니다. 배경색과 대비가 충분히 나는 밝은 색을 쓰세요.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13"/>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>수정 후: GitHub 저장소의 data/films.xlsx 를 이 파일로 교체해 올리면, 자동으로 data/films.json 이 만들어지고 사이트에 반영됩니다(1~3분).</t>
         </is>
@@ -838,7 +1095,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W51"/>
+  <dimension ref="A1:X51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -864,6 +1121,7 @@
     <col width="8" customWidth="1" min="21" max="21"/>
     <col width="11" customWidth="1" min="22" max="22"/>
     <col width="11" customWidth="1" min="23" max="23"/>
+    <col width="11" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -982,6 +1240,11 @@
           <t>배경색</t>
         </is>
       </c>
+      <c r="X1" s="5" t="inlineStr">
+        <is>
+          <t>포인트색</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -1089,6 +1352,11 @@
           <t>#2b2116</t>
         </is>
       </c>
+      <c r="X2" s="56" t="inlineStr">
+        <is>
+          <t>#e2b45c</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -1196,6 +1464,11 @@
           <t>#1d1c19</t>
         </is>
       </c>
+      <c r="X3" s="57" t="inlineStr">
+        <is>
+          <t>#e7c35a</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -1303,6 +1576,11 @@
           <t>#2a2017</t>
         </is>
       </c>
+      <c r="X4" s="58" t="inlineStr">
+        <is>
+          <t>#d9b88a</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -1410,6 +1688,11 @@
           <t>#1d2333</t>
         </is>
       </c>
+      <c r="X5" s="59" t="inlineStr">
+        <is>
+          <t>#f2ad96</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -1515,6 +1798,11 @@
       <c r="W6" s="10" t="inlineStr">
         <is>
           <t>#2c1215</t>
+        </is>
+      </c>
+      <c r="X6" s="60" t="inlineStr">
+        <is>
+          <t>#e3c27a</t>
         </is>
       </c>
     </row>
@@ -1620,6 +1908,11 @@
           <t>#241a0a</t>
         </is>
       </c>
+      <c r="X7" s="61" t="inlineStr">
+        <is>
+          <t>#f0b43c</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -1723,6 +2016,11 @@
           <t>#1c1a35</t>
         </is>
       </c>
+      <c r="X8" s="62" t="inlineStr">
+        <is>
+          <t>#f3cf6a</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -1826,6 +2124,11 @@
           <t>#2a140a</t>
         </is>
       </c>
+      <c r="X9" s="63" t="inlineStr">
+        <is>
+          <t>#f39a4b</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -1929,6 +2232,11 @@
           <t>#1a2b4f</t>
         </is>
       </c>
+      <c r="X10" s="64" t="inlineStr">
+        <is>
+          <t>#acccff</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -2032,6 +2340,11 @@
           <t>#1c2226</t>
         </is>
       </c>
+      <c r="X11" s="65" t="inlineStr">
+        <is>
+          <t>#b9c9d6</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -2139,6 +2452,11 @@
           <t>#1c1c1c</t>
         </is>
       </c>
+      <c r="X12" s="66" t="inlineStr">
+        <is>
+          <t>#cfcfcf</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -2246,6 +2564,11 @@
           <t>#1e1f17</t>
         </is>
       </c>
+      <c r="X13" s="67" t="inlineStr">
+        <is>
+          <t>#d4c48e</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -2351,6 +2674,11 @@
       <c r="W14" s="18" t="inlineStr">
         <is>
           <t>#1a2229</t>
+        </is>
+      </c>
+      <c r="X14" s="68" t="inlineStr">
+        <is>
+          <t>#a9cbe0</t>
         </is>
       </c>
     </row>
@@ -2456,6 +2784,11 @@
           <t>#10241a</t>
         </is>
       </c>
+      <c r="X15" s="69" t="inlineStr">
+        <is>
+          <t>#f9a491</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -2559,6 +2892,11 @@
           <t>#1c2230</t>
         </is>
       </c>
+      <c r="X16" s="70" t="inlineStr">
+        <is>
+          <t>#e6c79a</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -2662,6 +3000,11 @@
           <t>#1b1f1c</t>
         </is>
       </c>
+      <c r="X17" s="71" t="inlineStr">
+        <is>
+          <t>#b7c7a8</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -2765,6 +3108,11 @@
           <t>#0f2020</t>
         </is>
       </c>
+      <c r="X18" s="72" t="inlineStr">
+        <is>
+          <t>#d9b468</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -2868,6 +3216,11 @@
           <t>#2a1f17</t>
         </is>
       </c>
+      <c r="X19" s="73" t="inlineStr">
+        <is>
+          <t>#eab48a</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -2971,6 +3324,11 @@
           <t>#142219</t>
         </is>
       </c>
+      <c r="X20" s="74" t="inlineStr">
+        <is>
+          <t>#b8d98a</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -3074,6 +3432,11 @@
           <t>#1c2228</t>
         </is>
       </c>
+      <c r="X21" s="75" t="inlineStr">
+        <is>
+          <t>#c7d3dc</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -3179,6 +3542,11 @@
       <c r="W22" s="26" t="inlineStr">
         <is>
           <t>#2a1012</t>
+        </is>
+      </c>
+      <c r="X22" s="76" t="inlineStr">
+        <is>
+          <t>#f09a9a</t>
         </is>
       </c>
     </row>
@@ -3284,6 +3652,11 @@
           <t>#2e160b</t>
         </is>
       </c>
+      <c r="X23" s="77" t="inlineStr">
+        <is>
+          <t>#ff9a4a</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -3387,6 +3760,11 @@
           <t>#142030</t>
         </is>
       </c>
+      <c r="X24" s="78" t="inlineStr">
+        <is>
+          <t>#8fc3e6</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -3490,6 +3868,11 @@
           <t>#2a2015</t>
         </is>
       </c>
+      <c r="X25" s="79" t="inlineStr">
+        <is>
+          <t>#d8b47e</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -3593,6 +3976,11 @@
           <t>#0f151d</t>
         </is>
       </c>
+      <c r="X26" s="80" t="inlineStr">
+        <is>
+          <t>#8fb1d6</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -3696,6 +4084,11 @@
           <t>#15161c</t>
         </is>
       </c>
+      <c r="X27" s="81" t="inlineStr">
+        <is>
+          <t>#d8c79a</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
@@ -3799,6 +4192,11 @@
           <t>#1d1714</t>
         </is>
       </c>
+      <c r="X28" s="82" t="inlineStr">
+        <is>
+          <t>#f0a597</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -3902,6 +4300,11 @@
           <t>#1d2224</t>
         </is>
       </c>
+      <c r="X29" s="83" t="inlineStr">
+        <is>
+          <t>#b8c6c8</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
@@ -4005,6 +4408,11 @@
           <t>#1a2024</t>
         </is>
       </c>
+      <c r="X30" s="84" t="inlineStr">
+        <is>
+          <t>#a8c0cf</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -4108,6 +4516,11 @@
           <t>#2a1612</t>
         </is>
       </c>
+      <c r="X31" s="85" t="inlineStr">
+        <is>
+          <t>#e0b06a</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
@@ -4211,6 +4624,11 @@
           <t>#13253a</t>
         </is>
       </c>
+      <c r="X32" s="86" t="inlineStr">
+        <is>
+          <t>#f8ae9a</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
@@ -4314,6 +4732,11 @@
           <t>#12221a</t>
         </is>
       </c>
+      <c r="X33" s="87" t="inlineStr">
+        <is>
+          <t>#a9d08a</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
@@ -4421,6 +4844,11 @@
           <t>#2a1b10</t>
         </is>
       </c>
+      <c r="X34" s="88" t="inlineStr">
+        <is>
+          <t>#e8b878</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -4526,6 +4954,11 @@
       <c r="W35" s="39" t="inlineStr">
         <is>
           <t>#13203a</t>
+        </is>
+      </c>
+      <c r="X35" s="89" t="inlineStr">
+        <is>
+          <t>#f2c36b</t>
         </is>
       </c>
     </row>
@@ -4631,6 +5064,11 @@
           <t>#2a1030</t>
         </is>
       </c>
+      <c r="X36" s="90" t="inlineStr">
+        <is>
+          <t>#ffa6d0</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
@@ -4734,6 +5172,11 @@
           <t>#22143a</t>
         </is>
       </c>
+      <c r="X37" s="91" t="inlineStr">
+        <is>
+          <t>#ffb347</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
@@ -4837,6 +5280,11 @@
           <t>#17204a</t>
         </is>
       </c>
+      <c r="X38" s="92" t="inlineStr">
+        <is>
+          <t>#ffd75a</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
@@ -4940,6 +5388,11 @@
           <t>#2b2010</t>
         </is>
       </c>
+      <c r="X39" s="93" t="inlineStr">
+        <is>
+          <t>#f0c060</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
@@ -5043,6 +5496,11 @@
           <t>#1a1e45</t>
         </is>
       </c>
+      <c r="X40" s="94" t="inlineStr">
+        <is>
+          <t>#f5b39a</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
@@ -5146,6 +5604,11 @@
           <t>#13283a</t>
         </is>
       </c>
+      <c r="X41" s="95" t="inlineStr">
+        <is>
+          <t>#ffc96b</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
@@ -5249,6 +5712,11 @@
           <t>#18120d</t>
         </is>
       </c>
+      <c r="X42" s="96" t="inlineStr">
+        <is>
+          <t>#d4b06a</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
@@ -5352,6 +5820,11 @@
           <t>#142231</t>
         </is>
       </c>
+      <c r="X43" s="97" t="inlineStr">
+        <is>
+          <t>#c9d8e8</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
@@ -5455,6 +5928,11 @@
           <t>#2c1512</t>
         </is>
       </c>
+      <c r="X44" s="98" t="inlineStr">
+        <is>
+          <t>#f0c87a</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
@@ -5558,6 +6036,11 @@
           <t>#2a2016</t>
         </is>
       </c>
+      <c r="X45" s="99" t="inlineStr">
+        <is>
+          <t>#ecd08a</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
@@ -5661,6 +6144,11 @@
           <t>#26162f</t>
         </is>
       </c>
+      <c r="X46" s="100" t="inlineStr">
+        <is>
+          <t>#ffa84a</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
@@ -5764,6 +6252,11 @@
           <t>#24190f</t>
         </is>
       </c>
+      <c r="X47" s="101" t="inlineStr">
+        <is>
+          <t>#e3a96a</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
@@ -5867,6 +6360,11 @@
           <t>#1e1d16</t>
         </is>
       </c>
+      <c r="X48" s="102" t="inlineStr">
+        <is>
+          <t>#b9cc8a</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
@@ -5970,6 +6468,11 @@
           <t>#0f2522</t>
         </is>
       </c>
+      <c r="X49" s="103" t="inlineStr">
+        <is>
+          <t>#f2d45c</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
@@ -6073,6 +6576,11 @@
           <t>#222020</t>
         </is>
       </c>
+      <c r="X50" s="104" t="inlineStr">
+        <is>
+          <t>#eab0b0</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
@@ -6174,6 +6682,11 @@
       <c r="W51" s="55" t="inlineStr">
         <is>
           <t>#2b1210</t>
+        </is>
+      </c>
+      <c r="X51" s="105" t="inlineStr">
+        <is>
+          <t>#f2c94c</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Roma: yellow point colour, as on the poster
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q8auJtZCZpXRhnY2W8Jqqg
</commit_message>
<xml_diff>
--- a/data/films.xlsx
+++ b/data/films.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="54">
+  <fonts count="55">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -237,6 +237,10 @@
     <font>
       <b val="1"/>
       <color rgb="00f2c94c"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00f2d15a"/>
     </font>
   </fonts>
   <fills count="53">
@@ -514,7 +518,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="106">
+  <cellXfs count="107">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -627,6 +631,7 @@
     <xf numFmtId="0" fontId="51" fillId="50" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="52" fillId="51" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="53" fillId="52" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="54" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1005,7 +1010,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -1076,7 +1080,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
@@ -2452,9 +2455,9 @@
           <t>#1c1c1c</t>
         </is>
       </c>
-      <c r="X12" s="66" t="inlineStr">
-        <is>
-          <t>#cfcfcf</t>
+      <c r="X12" s="106" t="inlineStr">
+        <is>
+          <t>#f2d15a</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Poster colours: background and point colour from each poster
</commit_message>
<xml_diff>
--- a/data/films.xlsx
+++ b/data/films.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="사용법" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="추천작" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="제외작" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="사용법" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="추천작" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="제외작" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="55">
+  <fonts count="106">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -242,8 +242,210 @@
       <b val="1"/>
       <color rgb="00f2d15a"/>
     </font>
+    <font>
+      <color rgb="00000000"/>
+    </font>
+    <font>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00f9b189"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00fcaf91"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00cbbfc4"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00cbbfad"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00c9c577"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00feaba5"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00e0be75"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00d7bbb6"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00fcaf8b"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00c1c1c1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00c3c1b9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00bfc2cf"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="0073cdf1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00e8c636"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00c1bfcb"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00e9b977"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="0075ccf3"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00f1ba7d"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="0081d2a8"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00e0e5df"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00d2c072"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="005fd5d5"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00feb3a9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="0079cbf5"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00b6c3cb"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00e4e4e4"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00f9b288"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00aec4d6"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00f2c71b"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00f4b181"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00ffaea1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00fdb170"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00e4e5e0"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00a3c1fd"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00fdb190"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="008dd275"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00afbdfd"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="009ec2ff"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00feb3be"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00fcb177"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00ffae98"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00feb077"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00ffd38d"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00eac262"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00f6b270"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00c4bfc4"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00ddbc53"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00fdb1b8"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00f2dd3b"/>
+    </font>
   </fonts>
-  <fills count="53">
+  <fills count="202">
     <fill>
       <patternFill/>
     </fill>
@@ -503,6 +705,751 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="002b1210"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00eae0c8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="006b4b39"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00342d1d"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0022201c"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007e5a4c"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002f2e2a"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00e6e0d0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00332a2e"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00312e23"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00928877"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00655b4b"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00342d20"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="003d3a19"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00888548"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00312f14"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000f1215"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00b1272e"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002b2e31"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0037569d"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00856823"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001a2c53"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00db6c21"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00120302"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004b2004"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00231812"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00a45e3c"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00362b26"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00b0b1b5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00191919"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002d2e30"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00dcba44"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="006b6962"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00382d03"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00293641"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0006070f"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00242f38"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="009cb2af"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="006e8a96"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0022312f"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00036e2e"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00e8c636"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00073616"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00a87756"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00040308"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00462308"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001a201c"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00b18e5e"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002a2f2c"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000a1517"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="005394b1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00263032"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002f5e60"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="009a7c5c"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000c3436"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00171819"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="003c5849"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002d2e2f"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="003a4578"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00e0e5df"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00222a52"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00211010"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00988d5f"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00392929"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00f9d20c"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0019a1a2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00372d03"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002c647a"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00a42823"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00053343"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0091715b"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00070707"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="003f2817"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00000001"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00244e63"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00292e37"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00c1cdd2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="008e9aa2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00272f33"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001e1e1e"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00fdfdfd"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002e2e2e"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0023231d"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007f5841"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002e2e29"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00788d93"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00263947"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00213135"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00250f0a"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00f2c71b"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="003d2823"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ce6c54"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00d3b9a7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004d1d12"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="008c97a4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00b51b11"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00272f38"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00edc164"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00c17937"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="003c2b03"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0017120c"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00f9faf5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00322d27"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00f2439d"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004a71c7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00491b31"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00192651"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00d06939"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001f2b50"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001d194d"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0063a64b"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00282852"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00170d58"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="003e488c"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00252953"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0071a4d8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00325da6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00082f51"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002496d3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00af6874"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0000324b"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00070506"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00b87238"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00302d2e"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0012151c"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00bd9387"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002b2e34"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00010101"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00b2672a"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001b1712"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00e8d8c0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00312d29"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0004255b"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00eac262"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00162d53"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00e8a525"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ad6e29"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="003e2904"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00c48f7e"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00050305"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00462217"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00301512"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00cbaa3f"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="003f2623"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0053bcce"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00b74457"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0002343c"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00d12818"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00f4dd1f"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004d1c16"/>
       </patternFill>
     </fill>
   </fills>
@@ -518,7 +1465,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="107">
+  <cellXfs count="306">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -632,6 +1579,205 @@
     <xf numFmtId="0" fontId="52" fillId="51" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="53" fillId="52" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="54" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="55" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="57" fillId="55" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="53" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="54" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="58" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="58" fillId="58" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="56" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="57" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="61" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="59" fillId="61" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="59" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="60" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="64" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="60" fillId="64" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="62" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="63" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="67" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="61" fillId="67" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="65" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="66" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="70" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="62" fillId="70" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="68" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="69" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="73" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="63" fillId="73" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="71" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="72" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="76" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="64" fillId="76" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="74" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="75" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="79" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="65" fillId="79" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="77" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="78" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="82" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="66" fillId="82" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="80" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="81" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="85" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="67" fillId="85" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="83" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="84" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="88" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="68" fillId="88" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="86" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="87" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="91" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="69" fillId="91" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="89" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="90" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="94" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="70" fillId="94" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="92" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="93" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="97" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="71" fillId="97" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="95" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="96" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="100" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="72" fillId="100" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="98" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="99" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="103" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="73" fillId="103" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="101" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="102" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="106" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="74" fillId="106" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="104" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="105" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="109" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="75" fillId="109" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="107" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="108" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="112" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="76" fillId="112" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="110" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="111" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="115" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="77" fillId="115" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="113" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="114" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="118" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="78" fillId="118" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="116" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="117" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="121" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="79" fillId="121" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="119" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="120" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="124" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="66" fillId="124" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="122" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="123" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="127" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="80" fillId="127" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="125" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="126" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="130" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="81" fillId="130" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="128" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="129" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="133" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="82" fillId="133" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="131" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="132" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="136" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="83" fillId="136" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="134" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="135" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="139" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="84" fillId="139" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="137" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="138" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="142" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="142" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="140" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="141" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="145" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="86" fillId="145" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="143" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="144" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="148" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="87" fillId="148" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="146" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="147" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="151" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="88" fillId="151" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="149" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="150" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="154" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="89" fillId="154" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="152" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="153" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="157" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="90" fillId="157" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="155" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="156" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="160" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="91" fillId="160" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="158" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="159" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="163" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="92" fillId="163" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="161" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="162" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="166" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="93" fillId="166" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="164" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="165" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="169" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="94" fillId="169" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="167" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="168" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="172" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="95" fillId="172" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="170" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="171" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="175" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="96" fillId="175" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="173" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="174" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="178" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="97" fillId="178" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="176" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="177" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="98" fillId="133" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="179" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="180" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="183" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="99" fillId="183" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="181" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="182" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="186" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="100" fillId="186" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="184" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="185" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="189" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="101" fillId="189" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="187" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="188" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="192" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="102" fillId="192" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="190" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="191" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="195" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="103" fillId="195" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="193" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="194" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="198" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="104" fillId="198" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="196" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="197" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="201" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="105" fillId="201" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="199" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="200" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1098,7 +2244,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X51"/>
+  <dimension ref="A1:Z51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1125,6 +2271,8 @@
     <col width="11" customWidth="1" min="22" max="22"/>
     <col width="11" customWidth="1" min="23" max="23"/>
     <col width="11" customWidth="1" min="24" max="24"/>
+    <col width="11" customWidth="1" min="25" max="25"/>
+    <col width="11" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1248,6 +2396,16 @@
           <t>포인트색</t>
         </is>
       </c>
+      <c r="Y1" s="5" t="inlineStr">
+        <is>
+          <t>포스터1색</t>
+        </is>
+      </c>
+      <c r="Z1" s="5" t="inlineStr">
+        <is>
+          <t>포스터2색</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -1350,14 +2508,24 @@
           <t>elegant</t>
         </is>
       </c>
-      <c r="W2" s="6" t="inlineStr">
-        <is>
-          <t>#2b2116</t>
-        </is>
-      </c>
-      <c r="X2" s="56" t="inlineStr">
-        <is>
-          <t>#e2b45c</t>
+      <c r="W2" s="107" t="inlineStr">
+        <is>
+          <t>#342d1d</t>
+        </is>
+      </c>
+      <c r="X2" s="108" t="inlineStr">
+        <is>
+          <t>#f9b189</t>
+        </is>
+      </c>
+      <c r="Y2" s="109" t="inlineStr">
+        <is>
+          <t>#eae0c8</t>
+        </is>
+      </c>
+      <c r="Z2" s="110" t="inlineStr">
+        <is>
+          <t>#6b4b39</t>
         </is>
       </c>
     </row>
@@ -1462,14 +2630,24 @@
           <t>noir</t>
         </is>
       </c>
-      <c r="W3" s="7" t="inlineStr">
-        <is>
-          <t>#1d1c19</t>
-        </is>
-      </c>
-      <c r="X3" s="57" t="inlineStr">
-        <is>
-          <t>#e7c35a</t>
+      <c r="W3" s="111" t="inlineStr">
+        <is>
+          <t>#2f2e2a</t>
+        </is>
+      </c>
+      <c r="X3" s="112" t="inlineStr">
+        <is>
+          <t>#fcaf91</t>
+        </is>
+      </c>
+      <c r="Y3" s="113" t="inlineStr">
+        <is>
+          <t>#22201c</t>
+        </is>
+      </c>
+      <c r="Z3" s="114" t="inlineStr">
+        <is>
+          <t>#7e5a4c</t>
         </is>
       </c>
     </row>
@@ -1574,14 +2752,24 @@
           <t>western</t>
         </is>
       </c>
-      <c r="W4" s="8" t="inlineStr">
-        <is>
-          <t>#2a2017</t>
-        </is>
-      </c>
-      <c r="X4" s="58" t="inlineStr">
-        <is>
-          <t>#d9b88a</t>
+      <c r="W4" s="115" t="inlineStr">
+        <is>
+          <t>#312e23</t>
+        </is>
+      </c>
+      <c r="X4" s="116" t="inlineStr">
+        <is>
+          <t>#cbbfc4</t>
+        </is>
+      </c>
+      <c r="Y4" s="117" t="inlineStr">
+        <is>
+          <t>#e6e0d0</t>
+        </is>
+      </c>
+      <c r="Z4" s="118" t="inlineStr">
+        <is>
+          <t>#332a2e</t>
         </is>
       </c>
     </row>
@@ -1686,14 +2874,24 @@
           <t>typewriter</t>
         </is>
       </c>
-      <c r="W5" s="9" t="inlineStr">
-        <is>
-          <t>#1d2333</t>
-        </is>
-      </c>
-      <c r="X5" s="59" t="inlineStr">
-        <is>
-          <t>#f2ad96</t>
+      <c r="W5" s="119" t="inlineStr">
+        <is>
+          <t>#342d20</t>
+        </is>
+      </c>
+      <c r="X5" s="120" t="inlineStr">
+        <is>
+          <t>#cbbfad</t>
+        </is>
+      </c>
+      <c r="Y5" s="121" t="inlineStr">
+        <is>
+          <t>#928877</t>
+        </is>
+      </c>
+      <c r="Z5" s="122" t="inlineStr">
+        <is>
+          <t>#655b4b</t>
         </is>
       </c>
     </row>
@@ -1798,14 +2996,24 @@
           <t>epic</t>
         </is>
       </c>
-      <c r="W6" s="10" t="inlineStr">
-        <is>
-          <t>#2c1215</t>
-        </is>
-      </c>
-      <c r="X6" s="60" t="inlineStr">
-        <is>
-          <t>#e3c27a</t>
+      <c r="W6" s="123" t="inlineStr">
+        <is>
+          <t>#312f14</t>
+        </is>
+      </c>
+      <c r="X6" s="124" t="inlineStr">
+        <is>
+          <t>#c9c577</t>
+        </is>
+      </c>
+      <c r="Y6" s="125" t="inlineStr">
+        <is>
+          <t>#3d3a19</t>
+        </is>
+      </c>
+      <c r="Z6" s="126" t="inlineStr">
+        <is>
+          <t>#888548</t>
         </is>
       </c>
     </row>
@@ -1906,14 +3114,24 @@
           <t>bold</t>
         </is>
       </c>
-      <c r="W7" s="11" t="inlineStr">
-        <is>
-          <t>#241a0a</t>
-        </is>
-      </c>
-      <c r="X7" s="61" t="inlineStr">
-        <is>
-          <t>#f0b43c</t>
+      <c r="W7" s="127" t="inlineStr">
+        <is>
+          <t>#2b2e31</t>
+        </is>
+      </c>
+      <c r="X7" s="128" t="inlineStr">
+        <is>
+          <t>#feaba5</t>
+        </is>
+      </c>
+      <c r="Y7" s="129" t="inlineStr">
+        <is>
+          <t>#0f1215</t>
+        </is>
+      </c>
+      <c r="Z7" s="130" t="inlineStr">
+        <is>
+          <t>#b1272e</t>
         </is>
       </c>
     </row>
@@ -2014,14 +3232,24 @@
           <t>script</t>
         </is>
       </c>
-      <c r="W8" s="12" t="inlineStr">
-        <is>
-          <t>#1c1a35</t>
-        </is>
-      </c>
-      <c r="X8" s="62" t="inlineStr">
-        <is>
-          <t>#f3cf6a</t>
+      <c r="W8" s="131" t="inlineStr">
+        <is>
+          <t>#1a2c53</t>
+        </is>
+      </c>
+      <c r="X8" s="132" t="inlineStr">
+        <is>
+          <t>#e0be75</t>
+        </is>
+      </c>
+      <c r="Y8" s="133" t="inlineStr">
+        <is>
+          <t>#37569d</t>
+        </is>
+      </c>
+      <c r="Z8" s="134" t="inlineStr">
+        <is>
+          <t>#856823</t>
         </is>
       </c>
     </row>
@@ -2122,14 +3350,24 @@
           <t>bold</t>
         </is>
       </c>
-      <c r="W9" s="13" t="inlineStr">
-        <is>
-          <t>#2a140a</t>
-        </is>
-      </c>
-      <c r="X9" s="63" t="inlineStr">
-        <is>
-          <t>#f39a4b</t>
+      <c r="W9" s="135" t="inlineStr">
+        <is>
+          <t>#4b2004</t>
+        </is>
+      </c>
+      <c r="X9" s="136" t="inlineStr">
+        <is>
+          <t>#d7bbb6</t>
+        </is>
+      </c>
+      <c r="Y9" s="137" t="inlineStr">
+        <is>
+          <t>#db6c21</t>
+        </is>
+      </c>
+      <c r="Z9" s="138" t="inlineStr">
+        <is>
+          <t>#120302</t>
         </is>
       </c>
     </row>
@@ -2230,14 +3468,24 @@
           <t>mono</t>
         </is>
       </c>
-      <c r="W10" s="14" t="inlineStr">
-        <is>
-          <t>#1a2b4f</t>
-        </is>
-      </c>
-      <c r="X10" s="64" t="inlineStr">
-        <is>
-          <t>#acccff</t>
+      <c r="W10" s="139" t="inlineStr">
+        <is>
+          <t>#362b26</t>
+        </is>
+      </c>
+      <c r="X10" s="140" t="inlineStr">
+        <is>
+          <t>#fcaf8b</t>
+        </is>
+      </c>
+      <c r="Y10" s="141" t="inlineStr">
+        <is>
+          <t>#231812</t>
+        </is>
+      </c>
+      <c r="Z10" s="142" t="inlineStr">
+        <is>
+          <t>#a45e3c</t>
         </is>
       </c>
     </row>
@@ -2338,14 +3586,24 @@
           <t>typewriter</t>
         </is>
       </c>
-      <c r="W11" s="15" t="inlineStr">
-        <is>
-          <t>#1c2226</t>
-        </is>
-      </c>
-      <c r="X11" s="65" t="inlineStr">
-        <is>
-          <t>#b9c9d6</t>
+      <c r="W11" s="143" t="inlineStr">
+        <is>
+          <t>#2d2e30</t>
+        </is>
+      </c>
+      <c r="X11" s="144" t="inlineStr">
+        <is>
+          <t>#c1c1c1</t>
+        </is>
+      </c>
+      <c r="Y11" s="145" t="inlineStr">
+        <is>
+          <t>#b0b1b5</t>
+        </is>
+      </c>
+      <c r="Z11" s="146" t="inlineStr">
+        <is>
+          <t>#191919</t>
         </is>
       </c>
     </row>
@@ -2450,14 +3708,24 @@
           <t>elegant</t>
         </is>
       </c>
-      <c r="W12" s="16" t="inlineStr">
-        <is>
-          <t>#1c1c1c</t>
-        </is>
-      </c>
-      <c r="X12" s="106" t="inlineStr">
-        <is>
-          <t>#f2d15a</t>
+      <c r="W12" s="147" t="inlineStr">
+        <is>
+          <t>#382d03</t>
+        </is>
+      </c>
+      <c r="X12" s="148" t="inlineStr">
+        <is>
+          <t>#c3c1b9</t>
+        </is>
+      </c>
+      <c r="Y12" s="149" t="inlineStr">
+        <is>
+          <t>#dcba44</t>
+        </is>
+      </c>
+      <c r="Z12" s="150" t="inlineStr">
+        <is>
+          <t>#6b6962</t>
         </is>
       </c>
     </row>
@@ -2562,14 +3830,24 @@
           <t>epic</t>
         </is>
       </c>
-      <c r="W13" s="17" t="inlineStr">
-        <is>
-          <t>#1e1f17</t>
-        </is>
-      </c>
-      <c r="X13" s="67" t="inlineStr">
-        <is>
-          <t>#d4c48e</t>
+      <c r="W13" s="151" t="inlineStr">
+        <is>
+          <t>#242f38</t>
+        </is>
+      </c>
+      <c r="X13" s="152" t="inlineStr">
+        <is>
+          <t>#bfc2cf</t>
+        </is>
+      </c>
+      <c r="Y13" s="153" t="inlineStr">
+        <is>
+          <t>#293641</t>
+        </is>
+      </c>
+      <c r="Z13" s="154" t="inlineStr">
+        <is>
+          <t>#06070f</t>
         </is>
       </c>
     </row>
@@ -2674,14 +3952,24 @@
           <t>bold</t>
         </is>
       </c>
-      <c r="W14" s="18" t="inlineStr">
-        <is>
-          <t>#1a2229</t>
-        </is>
-      </c>
-      <c r="X14" s="68" t="inlineStr">
-        <is>
-          <t>#a9cbe0</t>
+      <c r="W14" s="155" t="inlineStr">
+        <is>
+          <t>#22312f</t>
+        </is>
+      </c>
+      <c r="X14" s="156" t="inlineStr">
+        <is>
+          <t>#73cdf1</t>
+        </is>
+      </c>
+      <c r="Y14" s="157" t="inlineStr">
+        <is>
+          <t>#9cb2af</t>
+        </is>
+      </c>
+      <c r="Z14" s="158" t="inlineStr">
+        <is>
+          <t>#6e8a96</t>
         </is>
       </c>
     </row>
@@ -2782,14 +4070,24 @@
           <t>hand</t>
         </is>
       </c>
-      <c r="W15" s="19" t="inlineStr">
-        <is>
-          <t>#10241a</t>
-        </is>
-      </c>
-      <c r="X15" s="69" t="inlineStr">
-        <is>
-          <t>#f9a491</t>
+      <c r="W15" s="159" t="inlineStr">
+        <is>
+          <t>#073616</t>
+        </is>
+      </c>
+      <c r="X15" s="160" t="inlineStr">
+        <is>
+          <t>#e8c636</t>
+        </is>
+      </c>
+      <c r="Y15" s="161" t="inlineStr">
+        <is>
+          <t>#036e2e</t>
+        </is>
+      </c>
+      <c r="Z15" s="162" t="inlineStr">
+        <is>
+          <t>#e8c636</t>
         </is>
       </c>
     </row>
@@ -2890,14 +4188,24 @@
           <t>bold</t>
         </is>
       </c>
-      <c r="W16" s="20" t="inlineStr">
-        <is>
-          <t>#1c2230</t>
-        </is>
-      </c>
-      <c r="X16" s="70" t="inlineStr">
-        <is>
-          <t>#e6c79a</t>
+      <c r="W16" s="163" t="inlineStr">
+        <is>
+          <t>#462308</t>
+        </is>
+      </c>
+      <c r="X16" s="164" t="inlineStr">
+        <is>
+          <t>#c1bfcb</t>
+        </is>
+      </c>
+      <c r="Y16" s="165" t="inlineStr">
+        <is>
+          <t>#a87756</t>
+        </is>
+      </c>
+      <c r="Z16" s="166" t="inlineStr">
+        <is>
+          <t>#040308</t>
         </is>
       </c>
     </row>
@@ -2998,14 +4306,24 @@
           <t>typewriter</t>
         </is>
       </c>
-      <c r="W17" s="21" t="inlineStr">
-        <is>
-          <t>#1b1f1c</t>
-        </is>
-      </c>
-      <c r="X17" s="71" t="inlineStr">
-        <is>
-          <t>#b7c7a8</t>
+      <c r="W17" s="167" t="inlineStr">
+        <is>
+          <t>#2a2f2c</t>
+        </is>
+      </c>
+      <c r="X17" s="168" t="inlineStr">
+        <is>
+          <t>#e9b977</t>
+        </is>
+      </c>
+      <c r="Y17" s="169" t="inlineStr">
+        <is>
+          <t>#1a201c</t>
+        </is>
+      </c>
+      <c r="Z17" s="170" t="inlineStr">
+        <is>
+          <t>#b18e5e</t>
         </is>
       </c>
     </row>
@@ -3106,14 +4424,24 @@
           <t>gothic</t>
         </is>
       </c>
-      <c r="W18" s="22" t="inlineStr">
-        <is>
-          <t>#0f2020</t>
-        </is>
-      </c>
-      <c r="X18" s="72" t="inlineStr">
-        <is>
-          <t>#d9b468</t>
+      <c r="W18" s="171" t="inlineStr">
+        <is>
+          <t>#263032</t>
+        </is>
+      </c>
+      <c r="X18" s="172" t="inlineStr">
+        <is>
+          <t>#75ccf3</t>
+        </is>
+      </c>
+      <c r="Y18" s="173" t="inlineStr">
+        <is>
+          <t>#0a1517</t>
+        </is>
+      </c>
+      <c r="Z18" s="174" t="inlineStr">
+        <is>
+          <t>#5394b1</t>
         </is>
       </c>
     </row>
@@ -3214,14 +4542,24 @@
           <t>elegant</t>
         </is>
       </c>
-      <c r="W19" s="23" t="inlineStr">
-        <is>
-          <t>#2a1f17</t>
-        </is>
-      </c>
-      <c r="X19" s="73" t="inlineStr">
-        <is>
-          <t>#eab48a</t>
+      <c r="W19" s="175" t="inlineStr">
+        <is>
+          <t>#0c3436</t>
+        </is>
+      </c>
+      <c r="X19" s="176" t="inlineStr">
+        <is>
+          <t>#f1ba7d</t>
+        </is>
+      </c>
+      <c r="Y19" s="177" t="inlineStr">
+        <is>
+          <t>#2f5e60</t>
+        </is>
+      </c>
+      <c r="Z19" s="178" t="inlineStr">
+        <is>
+          <t>#9a7c5c</t>
         </is>
       </c>
     </row>
@@ -3322,14 +4660,24 @@
           <t>retro</t>
         </is>
       </c>
-      <c r="W20" s="24" t="inlineStr">
-        <is>
-          <t>#142219</t>
-        </is>
-      </c>
-      <c r="X20" s="74" t="inlineStr">
-        <is>
-          <t>#b8d98a</t>
+      <c r="W20" s="179" t="inlineStr">
+        <is>
+          <t>#2d2e2f</t>
+        </is>
+      </c>
+      <c r="X20" s="180" t="inlineStr">
+        <is>
+          <t>#81d2a8</t>
+        </is>
+      </c>
+      <c r="Y20" s="181" t="inlineStr">
+        <is>
+          <t>#171819</t>
+        </is>
+      </c>
+      <c r="Z20" s="182" t="inlineStr">
+        <is>
+          <t>#3c5849</t>
         </is>
       </c>
     </row>
@@ -3430,14 +4778,24 @@
           <t>classic</t>
         </is>
       </c>
-      <c r="W21" s="25" t="inlineStr">
-        <is>
-          <t>#1c2228</t>
-        </is>
-      </c>
-      <c r="X21" s="75" t="inlineStr">
-        <is>
-          <t>#c7d3dc</t>
+      <c r="W21" s="183" t="inlineStr">
+        <is>
+          <t>#222a52</t>
+        </is>
+      </c>
+      <c r="X21" s="184" t="inlineStr">
+        <is>
+          <t>#e0e5df</t>
+        </is>
+      </c>
+      <c r="Y21" s="185" t="inlineStr">
+        <is>
+          <t>#3a4578</t>
+        </is>
+      </c>
+      <c r="Z21" s="186" t="inlineStr">
+        <is>
+          <t>#e0e5df</t>
         </is>
       </c>
     </row>
@@ -3542,14 +4900,24 @@
           <t>gothic</t>
         </is>
       </c>
-      <c r="W22" s="26" t="inlineStr">
-        <is>
-          <t>#2a1012</t>
-        </is>
-      </c>
-      <c r="X22" s="76" t="inlineStr">
-        <is>
-          <t>#f09a9a</t>
+      <c r="W22" s="187" t="inlineStr">
+        <is>
+          <t>#392929</t>
+        </is>
+      </c>
+      <c r="X22" s="188" t="inlineStr">
+        <is>
+          <t>#d2c072</t>
+        </is>
+      </c>
+      <c r="Y22" s="189" t="inlineStr">
+        <is>
+          <t>#211010</t>
+        </is>
+      </c>
+      <c r="Z22" s="190" t="inlineStr">
+        <is>
+          <t>#988d5f</t>
         </is>
       </c>
     </row>
@@ -3650,14 +5018,24 @@
           <t>bold</t>
         </is>
       </c>
-      <c r="W23" s="27" t="inlineStr">
-        <is>
-          <t>#2e160b</t>
-        </is>
-      </c>
-      <c r="X23" s="77" t="inlineStr">
-        <is>
-          <t>#ff9a4a</t>
+      <c r="W23" s="191" t="inlineStr">
+        <is>
+          <t>#372d03</t>
+        </is>
+      </c>
+      <c r="X23" s="192" t="inlineStr">
+        <is>
+          <t>#5fd5d5</t>
+        </is>
+      </c>
+      <c r="Y23" s="193" t="inlineStr">
+        <is>
+          <t>#f9d20c</t>
+        </is>
+      </c>
+      <c r="Z23" s="194" t="inlineStr">
+        <is>
+          <t>#19a1a2</t>
         </is>
       </c>
     </row>
@@ -3758,14 +5136,24 @@
           <t>scifi</t>
         </is>
       </c>
-      <c r="W24" s="28" t="inlineStr">
-        <is>
-          <t>#142030</t>
-        </is>
-      </c>
-      <c r="X24" s="78" t="inlineStr">
-        <is>
-          <t>#8fc3e6</t>
+      <c r="W24" s="195" t="inlineStr">
+        <is>
+          <t>#053343</t>
+        </is>
+      </c>
+      <c r="X24" s="196" t="inlineStr">
+        <is>
+          <t>#feb3a9</t>
+        </is>
+      </c>
+      <c r="Y24" s="197" t="inlineStr">
+        <is>
+          <t>#2c647a</t>
+        </is>
+      </c>
+      <c r="Z24" s="198" t="inlineStr">
+        <is>
+          <t>#a42823</t>
         </is>
       </c>
     </row>
@@ -3866,14 +5254,24 @@
           <t>western</t>
         </is>
       </c>
-      <c r="W25" s="29" t="inlineStr">
-        <is>
-          <t>#2a2015</t>
-        </is>
-      </c>
-      <c r="X25" s="79" t="inlineStr">
-        <is>
-          <t>#d8b47e</t>
+      <c r="W25" s="199" t="inlineStr">
+        <is>
+          <t>#3f2817</t>
+        </is>
+      </c>
+      <c r="X25" s="200" t="inlineStr">
+        <is>
+          <t>#c1c1c1</t>
+        </is>
+      </c>
+      <c r="Y25" s="201" t="inlineStr">
+        <is>
+          <t>#91715b</t>
+        </is>
+      </c>
+      <c r="Z25" s="202" t="inlineStr">
+        <is>
+          <t>#070707</t>
         </is>
       </c>
     </row>
@@ -3974,14 +5372,24 @@
           <t>bold</t>
         </is>
       </c>
-      <c r="W26" s="30" t="inlineStr">
-        <is>
-          <t>#0f151d</t>
-        </is>
-      </c>
-      <c r="X26" s="80" t="inlineStr">
-        <is>
-          <t>#8fb1d6</t>
+      <c r="W26" s="203" t="inlineStr">
+        <is>
+          <t>#292e37</t>
+        </is>
+      </c>
+      <c r="X26" s="204" t="inlineStr">
+        <is>
+          <t>#79cbf5</t>
+        </is>
+      </c>
+      <c r="Y26" s="205" t="inlineStr">
+        <is>
+          <t>#000001</t>
+        </is>
+      </c>
+      <c r="Z26" s="206" t="inlineStr">
+        <is>
+          <t>#244e63</t>
         </is>
       </c>
     </row>
@@ -4082,14 +5490,24 @@
           <t>scifi</t>
         </is>
       </c>
-      <c r="W27" s="31" t="inlineStr">
-        <is>
-          <t>#15161c</t>
-        </is>
-      </c>
-      <c r="X27" s="81" t="inlineStr">
-        <is>
-          <t>#d8c79a</t>
+      <c r="W27" s="207" t="inlineStr">
+        <is>
+          <t>#272f33</t>
+        </is>
+      </c>
+      <c r="X27" s="208" t="inlineStr">
+        <is>
+          <t>#b6c3cb</t>
+        </is>
+      </c>
+      <c r="Y27" s="209" t="inlineStr">
+        <is>
+          <t>#c1cdd2</t>
+        </is>
+      </c>
+      <c r="Z27" s="210" t="inlineStr">
+        <is>
+          <t>#8e9aa2</t>
         </is>
       </c>
     </row>
@@ -4190,14 +5608,24 @@
           <t>noir</t>
         </is>
       </c>
-      <c r="W28" s="32" t="inlineStr">
-        <is>
-          <t>#1d1714</t>
-        </is>
-      </c>
-      <c r="X28" s="82" t="inlineStr">
-        <is>
-          <t>#f0a597</t>
+      <c r="W28" s="211" t="inlineStr">
+        <is>
+          <t>#2e2e2e</t>
+        </is>
+      </c>
+      <c r="X28" s="212" t="inlineStr">
+        <is>
+          <t>#e4e4e4</t>
+        </is>
+      </c>
+      <c r="Y28" s="213" t="inlineStr">
+        <is>
+          <t>#1e1e1e</t>
+        </is>
+      </c>
+      <c r="Z28" s="214" t="inlineStr">
+        <is>
+          <t>#fdfdfd</t>
         </is>
       </c>
     </row>
@@ -4298,14 +5726,24 @@
           <t>light</t>
         </is>
       </c>
-      <c r="W29" s="33" t="inlineStr">
-        <is>
-          <t>#1d2224</t>
-        </is>
-      </c>
-      <c r="X29" s="83" t="inlineStr">
-        <is>
-          <t>#b8c6c8</t>
+      <c r="W29" s="215" t="inlineStr">
+        <is>
+          <t>#2e2e29</t>
+        </is>
+      </c>
+      <c r="X29" s="216" t="inlineStr">
+        <is>
+          <t>#f9b288</t>
+        </is>
+      </c>
+      <c r="Y29" s="217" t="inlineStr">
+        <is>
+          <t>#23231d</t>
+        </is>
+      </c>
+      <c r="Z29" s="218" t="inlineStr">
+        <is>
+          <t>#7f5841</t>
         </is>
       </c>
     </row>
@@ -4406,14 +5844,24 @@
           <t>noir</t>
         </is>
       </c>
-      <c r="W30" s="34" t="inlineStr">
-        <is>
-          <t>#1a2024</t>
-        </is>
-      </c>
-      <c r="X30" s="84" t="inlineStr">
-        <is>
-          <t>#a8c0cf</t>
+      <c r="W30" s="219" t="inlineStr">
+        <is>
+          <t>#213135</t>
+        </is>
+      </c>
+      <c r="X30" s="220" t="inlineStr">
+        <is>
+          <t>#aec4d6</t>
+        </is>
+      </c>
+      <c r="Y30" s="221" t="inlineStr">
+        <is>
+          <t>#788d93</t>
+        </is>
+      </c>
+      <c r="Z30" s="222" t="inlineStr">
+        <is>
+          <t>#263947</t>
         </is>
       </c>
     </row>
@@ -4514,14 +5962,24 @@
           <t>classic</t>
         </is>
       </c>
-      <c r="W31" s="35" t="inlineStr">
-        <is>
-          <t>#2a1612</t>
-        </is>
-      </c>
-      <c r="X31" s="85" t="inlineStr">
-        <is>
-          <t>#e0b06a</t>
+      <c r="W31" s="223" t="inlineStr">
+        <is>
+          <t>#3d2823</t>
+        </is>
+      </c>
+      <c r="X31" s="224" t="inlineStr">
+        <is>
+          <t>#f2c71b</t>
+        </is>
+      </c>
+      <c r="Y31" s="225" t="inlineStr">
+        <is>
+          <t>#250f0a</t>
+        </is>
+      </c>
+      <c r="Z31" s="226" t="inlineStr">
+        <is>
+          <t>#f2c71b</t>
         </is>
       </c>
     </row>
@@ -4622,14 +6080,24 @@
           <t>hand</t>
         </is>
       </c>
-      <c r="W32" s="36" t="inlineStr">
-        <is>
-          <t>#13253a</t>
-        </is>
-      </c>
-      <c r="X32" s="86" t="inlineStr">
-        <is>
-          <t>#f8ae9a</t>
+      <c r="W32" s="227" t="inlineStr">
+        <is>
+          <t>#4d1d12</t>
+        </is>
+      </c>
+      <c r="X32" s="228" t="inlineStr">
+        <is>
+          <t>#f4b181</t>
+        </is>
+      </c>
+      <c r="Y32" s="229" t="inlineStr">
+        <is>
+          <t>#ce6c54</t>
+        </is>
+      </c>
+      <c r="Z32" s="230" t="inlineStr">
+        <is>
+          <t>#d3b9a7</t>
         </is>
       </c>
     </row>
@@ -4730,14 +6198,24 @@
           <t>epic</t>
         </is>
       </c>
-      <c r="W33" s="37" t="inlineStr">
-        <is>
-          <t>#12221a</t>
-        </is>
-      </c>
-      <c r="X33" s="87" t="inlineStr">
-        <is>
-          <t>#a9d08a</t>
+      <c r="W33" s="231" t="inlineStr">
+        <is>
+          <t>#272f38</t>
+        </is>
+      </c>
+      <c r="X33" s="232" t="inlineStr">
+        <is>
+          <t>#ffaea1</t>
+        </is>
+      </c>
+      <c r="Y33" s="233" t="inlineStr">
+        <is>
+          <t>#8c97a4</t>
+        </is>
+      </c>
+      <c r="Z33" s="234" t="inlineStr">
+        <is>
+          <t>#b51b11</t>
         </is>
       </c>
     </row>
@@ -4842,14 +6320,24 @@
           <t>script</t>
         </is>
       </c>
-      <c r="W34" s="38" t="inlineStr">
-        <is>
-          <t>#2a1b10</t>
-        </is>
-      </c>
-      <c r="X34" s="88" t="inlineStr">
-        <is>
-          <t>#e8b878</t>
+      <c r="W34" s="235" t="inlineStr">
+        <is>
+          <t>#3c2b03</t>
+        </is>
+      </c>
+      <c r="X34" s="236" t="inlineStr">
+        <is>
+          <t>#fdb170</t>
+        </is>
+      </c>
+      <c r="Y34" s="237" t="inlineStr">
+        <is>
+          <t>#edc164</t>
+        </is>
+      </c>
+      <c r="Z34" s="238" t="inlineStr">
+        <is>
+          <t>#c17937</t>
         </is>
       </c>
     </row>
@@ -4954,14 +6442,24 @@
           <t>hand</t>
         </is>
       </c>
-      <c r="W35" s="39" t="inlineStr">
-        <is>
-          <t>#13203a</t>
-        </is>
-      </c>
-      <c r="X35" s="89" t="inlineStr">
-        <is>
-          <t>#f2c36b</t>
+      <c r="W35" s="239" t="inlineStr">
+        <is>
+          <t>#322d27</t>
+        </is>
+      </c>
+      <c r="X35" s="240" t="inlineStr">
+        <is>
+          <t>#e4e5e0</t>
+        </is>
+      </c>
+      <c r="Y35" s="241" t="inlineStr">
+        <is>
+          <t>#17120c</t>
+        </is>
+      </c>
+      <c r="Z35" s="242" t="inlineStr">
+        <is>
+          <t>#f9faf5</t>
         </is>
       </c>
     </row>
@@ -5062,14 +6560,24 @@
           <t>comic</t>
         </is>
       </c>
-      <c r="W36" s="40" t="inlineStr">
-        <is>
-          <t>#2a1030</t>
-        </is>
-      </c>
-      <c r="X36" s="90" t="inlineStr">
-        <is>
-          <t>#ffa6d0</t>
+      <c r="W36" s="243" t="inlineStr">
+        <is>
+          <t>#491b31</t>
+        </is>
+      </c>
+      <c r="X36" s="244" t="inlineStr">
+        <is>
+          <t>#a3c1fd</t>
+        </is>
+      </c>
+      <c r="Y36" s="245" t="inlineStr">
+        <is>
+          <t>#f2439d</t>
+        </is>
+      </c>
+      <c r="Z36" s="246" t="inlineStr">
+        <is>
+          <t>#4a71c7</t>
         </is>
       </c>
     </row>
@@ -5170,14 +6678,24 @@
           <t>script</t>
         </is>
       </c>
-      <c r="W37" s="41" t="inlineStr">
-        <is>
-          <t>#22143a</t>
-        </is>
-      </c>
-      <c r="X37" s="91" t="inlineStr">
-        <is>
-          <t>#ffb347</t>
+      <c r="W37" s="247" t="inlineStr">
+        <is>
+          <t>#1f2b50</t>
+        </is>
+      </c>
+      <c r="X37" s="248" t="inlineStr">
+        <is>
+          <t>#fdb190</t>
+        </is>
+      </c>
+      <c r="Y37" s="249" t="inlineStr">
+        <is>
+          <t>#192651</t>
+        </is>
+      </c>
+      <c r="Z37" s="250" t="inlineStr">
+        <is>
+          <t>#d06939</t>
         </is>
       </c>
     </row>
@@ -5278,14 +6796,24 @@
           <t>hand</t>
         </is>
       </c>
-      <c r="W38" s="42" t="inlineStr">
-        <is>
-          <t>#17204a</t>
-        </is>
-      </c>
-      <c r="X38" s="92" t="inlineStr">
-        <is>
-          <t>#ffd75a</t>
+      <c r="W38" s="251" t="inlineStr">
+        <is>
+          <t>#282852</t>
+        </is>
+      </c>
+      <c r="X38" s="252" t="inlineStr">
+        <is>
+          <t>#8dd275</t>
+        </is>
+      </c>
+      <c r="Y38" s="253" t="inlineStr">
+        <is>
+          <t>#1d194d</t>
+        </is>
+      </c>
+      <c r="Z38" s="254" t="inlineStr">
+        <is>
+          <t>#63a64b</t>
         </is>
       </c>
     </row>
@@ -5386,14 +6914,24 @@
           <t>scifi</t>
         </is>
       </c>
-      <c r="W39" s="43" t="inlineStr">
-        <is>
-          <t>#2b2010</t>
-        </is>
-      </c>
-      <c r="X39" s="93" t="inlineStr">
-        <is>
-          <t>#f0c060</t>
+      <c r="W39" s="255" t="inlineStr">
+        <is>
+          <t>#252953</t>
+        </is>
+      </c>
+      <c r="X39" s="256" t="inlineStr">
+        <is>
+          <t>#afbdfd</t>
+        </is>
+      </c>
+      <c r="Y39" s="257" t="inlineStr">
+        <is>
+          <t>#170d58</t>
+        </is>
+      </c>
+      <c r="Z39" s="258" t="inlineStr">
+        <is>
+          <t>#3e488c</t>
         </is>
       </c>
     </row>
@@ -5494,14 +7032,24 @@
           <t>light</t>
         </is>
       </c>
-      <c r="W40" s="44" t="inlineStr">
-        <is>
-          <t>#1a1e45</t>
-        </is>
-      </c>
-      <c r="X40" s="94" t="inlineStr">
-        <is>
-          <t>#f5b39a</t>
+      <c r="W40" s="259" t="inlineStr">
+        <is>
+          <t>#082f51</t>
+        </is>
+      </c>
+      <c r="X40" s="260" t="inlineStr">
+        <is>
+          <t>#9ec2ff</t>
+        </is>
+      </c>
+      <c r="Y40" s="261" t="inlineStr">
+        <is>
+          <t>#71a4d8</t>
+        </is>
+      </c>
+      <c r="Z40" s="262" t="inlineStr">
+        <is>
+          <t>#325da6</t>
         </is>
       </c>
     </row>
@@ -5602,14 +7150,24 @@
           <t>retro</t>
         </is>
       </c>
-      <c r="W41" s="45" t="inlineStr">
-        <is>
-          <t>#13283a</t>
-        </is>
-      </c>
-      <c r="X41" s="95" t="inlineStr">
-        <is>
-          <t>#ffc96b</t>
+      <c r="W41" s="263" t="inlineStr">
+        <is>
+          <t>#00324b</t>
+        </is>
+      </c>
+      <c r="X41" s="264" t="inlineStr">
+        <is>
+          <t>#feb3be</t>
+        </is>
+      </c>
+      <c r="Y41" s="265" t="inlineStr">
+        <is>
+          <t>#2496d3</t>
+        </is>
+      </c>
+      <c r="Z41" s="266" t="inlineStr">
+        <is>
+          <t>#af6874</t>
         </is>
       </c>
     </row>
@@ -5710,14 +7268,24 @@
           <t>noir</t>
         </is>
       </c>
-      <c r="W42" s="46" t="inlineStr">
-        <is>
-          <t>#18120d</t>
-        </is>
-      </c>
-      <c r="X42" s="96" t="inlineStr">
-        <is>
-          <t>#d4b06a</t>
+      <c r="W42" s="267" t="inlineStr">
+        <is>
+          <t>#302d2e</t>
+        </is>
+      </c>
+      <c r="X42" s="268" t="inlineStr">
+        <is>
+          <t>#fcb177</t>
+        </is>
+      </c>
+      <c r="Y42" s="269" t="inlineStr">
+        <is>
+          <t>#070506</t>
+        </is>
+      </c>
+      <c r="Z42" s="270" t="inlineStr">
+        <is>
+          <t>#b87238</t>
         </is>
       </c>
     </row>
@@ -5818,14 +7386,24 @@
           <t>typewriter</t>
         </is>
       </c>
-      <c r="W43" s="47" t="inlineStr">
-        <is>
-          <t>#142231</t>
-        </is>
-      </c>
-      <c r="X43" s="97" t="inlineStr">
-        <is>
-          <t>#c9d8e8</t>
+      <c r="W43" s="271" t="inlineStr">
+        <is>
+          <t>#2b2e34</t>
+        </is>
+      </c>
+      <c r="X43" s="272" t="inlineStr">
+        <is>
+          <t>#ffae98</t>
+        </is>
+      </c>
+      <c r="Y43" s="273" t="inlineStr">
+        <is>
+          <t>#12151c</t>
+        </is>
+      </c>
+      <c r="Z43" s="274" t="inlineStr">
+        <is>
+          <t>#bd9387</t>
         </is>
       </c>
     </row>
@@ -5926,14 +7504,24 @@
           <t>script</t>
         </is>
       </c>
-      <c r="W44" s="48" t="inlineStr">
-        <is>
-          <t>#2c1512</t>
-        </is>
-      </c>
-      <c r="X44" s="98" t="inlineStr">
-        <is>
-          <t>#f0c87a</t>
+      <c r="W44" s="211" t="inlineStr">
+        <is>
+          <t>#2e2e2e</t>
+        </is>
+      </c>
+      <c r="X44" s="275" t="inlineStr">
+        <is>
+          <t>#feb077</t>
+        </is>
+      </c>
+      <c r="Y44" s="276" t="inlineStr">
+        <is>
+          <t>#010101</t>
+        </is>
+      </c>
+      <c r="Z44" s="277" t="inlineStr">
+        <is>
+          <t>#b2672a</t>
         </is>
       </c>
     </row>
@@ -6034,14 +7622,24 @@
           <t>elegant</t>
         </is>
       </c>
-      <c r="W45" s="49" t="inlineStr">
-        <is>
-          <t>#2a2016</t>
-        </is>
-      </c>
-      <c r="X45" s="99" t="inlineStr">
-        <is>
-          <t>#ecd08a</t>
+      <c r="W45" s="278" t="inlineStr">
+        <is>
+          <t>#312d29</t>
+        </is>
+      </c>
+      <c r="X45" s="279" t="inlineStr">
+        <is>
+          <t>#ffd38d</t>
+        </is>
+      </c>
+      <c r="Y45" s="280" t="inlineStr">
+        <is>
+          <t>#1b1712</t>
+        </is>
+      </c>
+      <c r="Z45" s="281" t="inlineStr">
+        <is>
+          <t>#e8d8c0</t>
         </is>
       </c>
     </row>
@@ -6142,14 +7740,24 @@
           <t>retro</t>
         </is>
       </c>
-      <c r="W46" s="50" t="inlineStr">
-        <is>
-          <t>#26162f</t>
-        </is>
-      </c>
-      <c r="X46" s="100" t="inlineStr">
-        <is>
-          <t>#ffa84a</t>
+      <c r="W46" s="282" t="inlineStr">
+        <is>
+          <t>#162d53</t>
+        </is>
+      </c>
+      <c r="X46" s="283" t="inlineStr">
+        <is>
+          <t>#eac262</t>
+        </is>
+      </c>
+      <c r="Y46" s="284" t="inlineStr">
+        <is>
+          <t>#04255b</t>
+        </is>
+      </c>
+      <c r="Z46" s="285" t="inlineStr">
+        <is>
+          <t>#eac262</t>
         </is>
       </c>
     </row>
@@ -6250,14 +7858,24 @@
           <t>light</t>
         </is>
       </c>
-      <c r="W47" s="51" t="inlineStr">
-        <is>
-          <t>#24190f</t>
-        </is>
-      </c>
-      <c r="X47" s="101" t="inlineStr">
-        <is>
-          <t>#e3a96a</t>
+      <c r="W47" s="286" t="inlineStr">
+        <is>
+          <t>#3e2904</t>
+        </is>
+      </c>
+      <c r="X47" s="287" t="inlineStr">
+        <is>
+          <t>#f6b270</t>
+        </is>
+      </c>
+      <c r="Y47" s="288" t="inlineStr">
+        <is>
+          <t>#e8a525</t>
+        </is>
+      </c>
+      <c r="Z47" s="289" t="inlineStr">
+        <is>
+          <t>#ad6e29</t>
         </is>
       </c>
     </row>
@@ -6358,14 +7976,24 @@
           <t>bold</t>
         </is>
       </c>
-      <c r="W48" s="52" t="inlineStr">
-        <is>
-          <t>#1e1d16</t>
-        </is>
-      </c>
-      <c r="X48" s="102" t="inlineStr">
-        <is>
-          <t>#b9cc8a</t>
+      <c r="W48" s="290" t="inlineStr">
+        <is>
+          <t>#462217</t>
+        </is>
+      </c>
+      <c r="X48" s="291" t="inlineStr">
+        <is>
+          <t>#c4bfc4</t>
+        </is>
+      </c>
+      <c r="Y48" s="292" t="inlineStr">
+        <is>
+          <t>#c48f7e</t>
+        </is>
+      </c>
+      <c r="Z48" s="293" t="inlineStr">
+        <is>
+          <t>#050305</t>
         </is>
       </c>
     </row>
@@ -6466,14 +8094,24 @@
           <t>neon</t>
         </is>
       </c>
-      <c r="W49" s="53" t="inlineStr">
-        <is>
-          <t>#0f2522</t>
-        </is>
-      </c>
-      <c r="X49" s="103" t="inlineStr">
-        <is>
-          <t>#f2d45c</t>
+      <c r="W49" s="294" t="inlineStr">
+        <is>
+          <t>#3f2623</t>
+        </is>
+      </c>
+      <c r="X49" s="295" t="inlineStr">
+        <is>
+          <t>#ddbc53</t>
+        </is>
+      </c>
+      <c r="Y49" s="296" t="inlineStr">
+        <is>
+          <t>#301512</t>
+        </is>
+      </c>
+      <c r="Z49" s="297" t="inlineStr">
+        <is>
+          <t>#cbaa3f</t>
         </is>
       </c>
     </row>
@@ -6574,14 +8212,24 @@
           <t>script</t>
         </is>
       </c>
-      <c r="W50" s="54" t="inlineStr">
-        <is>
-          <t>#222020</t>
-        </is>
-      </c>
-      <c r="X50" s="104" t="inlineStr">
-        <is>
-          <t>#eab0b0</t>
+      <c r="W50" s="298" t="inlineStr">
+        <is>
+          <t>#02343c</t>
+        </is>
+      </c>
+      <c r="X50" s="299" t="inlineStr">
+        <is>
+          <t>#fdb1b8</t>
+        </is>
+      </c>
+      <c r="Y50" s="300" t="inlineStr">
+        <is>
+          <t>#53bcce</t>
+        </is>
+      </c>
+      <c r="Z50" s="301" t="inlineStr">
+        <is>
+          <t>#b74457</t>
         </is>
       </c>
     </row>
@@ -6682,14 +8330,24 @@
           <t>retro</t>
         </is>
       </c>
-      <c r="W51" s="55" t="inlineStr">
-        <is>
-          <t>#2b1210</t>
-        </is>
-      </c>
-      <c r="X51" s="105" t="inlineStr">
-        <is>
-          <t>#f2c94c</t>
+      <c r="W51" s="302" t="inlineStr">
+        <is>
+          <t>#4d1c16</t>
+        </is>
+      </c>
+      <c r="X51" s="303" t="inlineStr">
+        <is>
+          <t>#f2dd3b</t>
+        </is>
+      </c>
+      <c r="Y51" s="304" t="inlineStr">
+        <is>
+          <t>#d12818</t>
+        </is>
+      </c>
+      <c r="Z51" s="305" t="inlineStr">
+        <is>
+          <t>#f4dd1f</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Poster colours: try other posters for weak palettes, 선호색 hint, 포스터 override
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q8auJtZCZpXRhnY2W8Jqqg
</commit_message>
<xml_diff>
--- a/data/films.xlsx
+++ b/data/films.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="사용법" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="추천작" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="제외작" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="사용법" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="추천작" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="제외작" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3648,7 +3648,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -3735,6 +3735,20 @@
       <c r="A14" t="inlineStr">
         <is>
           <t>수정 후: GitHub 저장소의 data/films.xlsx 를 이 파일로 교체해 올리면, 자동으로 data/films.json 이 만들어지고 사이트에 반영됩니다(1~3분).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>11. 포스터: 색 분석으로 더 잘 어울리는 포스터를 고른 경우 그 TMDB 이미지 경로가 들어갑니다. 비우면 기본 포스터를 씁니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>12. 선호색: 상세 페이지에 꼭 들어갔으면 하는 색(빨강·주황·노랑·초록·청록·파랑·남색·보라·분홍). 'Poster colours' 실행 때 그 색이 있는 포스터를 찾아 씁니다.</t>
         </is>
       </c>
     </row>
@@ -3749,7 +3763,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z51"/>
+  <dimension ref="A1:AB51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3778,6 +3792,8 @@
     <col width="11" customWidth="1" min="24" max="24"/>
     <col width="11" customWidth="1" min="25" max="25"/>
     <col width="11" customWidth="1" min="26" max="26"/>
+    <col width="30" customWidth="1" min="27" max="27"/>
+    <col width="14" customWidth="1" min="28" max="28"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3911,6 +3927,16 @@
           <t>포스터2색</t>
         </is>
       </c>
+      <c r="AA1" s="5" t="inlineStr">
+        <is>
+          <t>포스터</t>
+        </is>
+      </c>
+      <c r="AB1" s="5" t="inlineStr">
+        <is>
+          <t>선호색</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -4991,6 +5017,11 @@
       <c r="Z10" s="142" t="inlineStr">
         <is>
           <t>#a45e3c</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>파랑</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Poster colours: preferred colour becomes the page background
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q8auJtZCZpXRhnY2W8Jqqg
</commit_message>
<xml_diff>
--- a/data/films.xlsx
+++ b/data/films.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="사용법" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="추천작" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="제외작" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="사용법" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="추천작" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="제외작" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4226,6 +4226,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -4296,6 +4297,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
@@ -4313,7 +4315,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>12. 선호색: 상세 페이지에 꼭 들어갔으면 하는 색(빨강·주황·노랑·초록·청록·파랑·남색·보라·분홍). 'Poster colours' 실행 때 그 색이 있는 포스터를 찾아 씁니다.</t>
+          <t>12. 선호색: 상세 페이지 배경으로 쓰고 싶은 색(빨강·주황·노랑·초록·청록·파랑·남색·보라·분홍). 'Poster colours' 실행 때 그 색이 있는 포스터를 찾아 배경색으로 쓰고, 어울리는 포인트색을 고릅니다.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Marriage Story: shirt colours (mauve-brown base, brick point); 색고정 lock
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q8auJtZCZpXRhnY2W8Jqqg
</commit_message>
<xml_diff>
--- a/data/films.xlsx
+++ b/data/films.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="사용법" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="추천작" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="제외작" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="사용법" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="추천작" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="제외작" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="228">
+  <fonts count="229">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -932,8 +932,12 @@
       <b val="1"/>
       <color rgb="00ee694f"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00d57769"/>
+    </font>
   </fonts>
-  <fills count="447">
+  <fills count="450">
     <fill>
       <patternFill/>
     </fill>
@@ -3161,6 +3165,21 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00b9381f"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0055403a"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00823c32"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0032221d"/>
       </patternFill>
     </fill>
   </fills>
@@ -3176,7 +3195,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="682">
+  <cellXfs count="686">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -3865,6 +3884,10 @@
     <xf numFmtId="0" fontId="227" fillId="410" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="56" fillId="446" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="100" fillId="318" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="449" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="228" fillId="449" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="447" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="448" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -4230,7 +4253,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -4331,6 +4354,13 @@
       <c r="A16" t="inlineStr">
         <is>
           <t>12. 선호색: 상세 페이지 배경으로 쓰고 싶은 색(빨강·주황·노랑·초록·청록·파랑·남색·보라·분홍). 'Poster colours' 실행 때 그 색이 있는 포스터를 찾아 배경색으로 쓰고, 어울리는 포인트색을 고릅니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>13. 색고정: O로 표시한 영화는 'Poster colours'를 다시 실행해도 배경색·포인트색·포스터를 바꾸지 않습니다(직접 지정한 색 보호).</t>
         </is>
       </c>
     </row>
@@ -4345,7 +4375,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB51"/>
+  <dimension ref="A1:AC51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4376,6 +4406,7 @@
     <col width="11" customWidth="1" min="26" max="26"/>
     <col width="30" customWidth="1" min="27" max="27"/>
     <col width="14" customWidth="1" min="28" max="28"/>
+    <col width="8" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4519,6 +4550,11 @@
           <t>선호색</t>
         </is>
       </c>
+      <c r="AC1" s="5" t="inlineStr">
+        <is>
+          <t>색고정</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -4621,29 +4657,34 @@
           <t>elegant</t>
         </is>
       </c>
-      <c r="W2" s="577" t="inlineStr">
-        <is>
-          <t>#3d1c0c</t>
-        </is>
-      </c>
-      <c r="X2" s="578" t="inlineStr">
-        <is>
-          <t>#d88754</t>
-        </is>
-      </c>
-      <c r="Y2" s="579" t="inlineStr">
-        <is>
-          <t>#754a35</t>
-        </is>
-      </c>
-      <c r="Z2" s="580" t="inlineStr">
-        <is>
-          <t>#bc947d</t>
+      <c r="W2" s="682" t="inlineStr">
+        <is>
+          <t>#32221d</t>
+        </is>
+      </c>
+      <c r="X2" s="683" t="inlineStr">
+        <is>
+          <t>#d57769</t>
+        </is>
+      </c>
+      <c r="Y2" s="684" t="inlineStr">
+        <is>
+          <t>#55403a</t>
+        </is>
+      </c>
+      <c r="Z2" s="685" t="inlineStr">
+        <is>
+          <t>#823c32</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
         <is>
           <t>/tySBjF6ixqASkG3MnIiF6fTxGPm.jpg</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Match posters to the chosen references
</commit_message>
<xml_diff>
--- a/data/films.xlsx
+++ b/data/films.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="사용법" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="추천작" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="제외작" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="사용법" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="추천작" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="제외작" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4811,7 +4811,7 @@
       </c>
       <c r="AA3" t="inlineStr">
         <is>
-          <t>/hayIQUwGjlKu5sfkHdnocIy7HI9.jpg</t>
+          <t>/mbm8k3GFhXS0ROd9AD1gqYbIFbM.jpg</t>
         </is>
       </c>
     </row>
@@ -5060,7 +5060,7 @@
       </c>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>/iUTe9RXZDog3f7wAF2aEIuXfNzc.jpg</t>
+          <t>/fK4l8KyVZAPlEJ9oUxblz70Qeyy.jpg</t>
         </is>
       </c>
     </row>
@@ -5185,6 +5185,11 @@
           <t>#888548</t>
         </is>
       </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>/4d4mTSfDIFIbUbMLUfaKodvxYXA.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -5303,6 +5308,11 @@
           <t>#b1272e</t>
         </is>
       </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>/7fn624j5lj3xTme2SgiLCeuedmO.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -5421,6 +5431,11 @@
           <t>#856823</t>
         </is>
       </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>/lcYwCSTzCHv0Z2QRpfztt75JyYj.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -5539,6 +5554,11 @@
           <t>#deb767</t>
         </is>
       </c>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>/jtTHxuJhuZpFAnCI4vGjg1LGmpY.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -5659,7 +5679,7 @@
       </c>
       <c r="AA10" t="inlineStr">
         <is>
-          <t>/7zqCN76W9pUc4EwmZm5neEXRa2M.jpg</t>
+          <t>/n0ybibhJtQ5icDqTp8eRytcIHJx.jpg</t>
         </is>
       </c>
       <c r="AB10" t="inlineStr">
@@ -6163,7 +6183,7 @@
       </c>
       <c r="AA14" t="inlineStr">
         <is>
-          <t>/yTWJd1v7CJ30w9yW7buEinbSlxV.jpg</t>
+          <t>/2e853FDVSIso600RqAMunPxiZjq.jpg</t>
         </is>
       </c>
     </row>
@@ -6402,6 +6422,11 @@
           <t>#a87756</t>
         </is>
       </c>
+      <c r="AA16" t="inlineStr">
+        <is>
+          <t>/f6ORXXQdIKHU3RvC6AC2lwAD6Mq.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -6522,7 +6547,7 @@
       </c>
       <c r="AA17" t="inlineStr">
         <is>
-          <t>/24PDYTAr7xSAVL7Aw275MoqnpAd.jpg</t>
+          <t>/cVUDMnskSc01rdbyH0tLATTJUdP.jpg</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6670,7 @@
       </c>
       <c r="AA18" t="inlineStr">
         <is>
-          <t>/2VVhikIxoztAXEDQZLOdtBsu6vf.jpg</t>
+          <t>/s8C4whhKtDaJvMDcyiMvx3BIF5F.jpg</t>
         </is>
       </c>
     </row>
@@ -6768,7 +6793,7 @@
       </c>
       <c r="AA19" t="inlineStr">
         <is>
-          <t>/1vlgCjejhux4P5TcRJlZOk739Hr.jpg</t>
+          <t>/11zlNdxiHhhW5BWgL2PkqaRCzTM.jpg</t>
         </is>
       </c>
     </row>
@@ -7014,7 +7039,7 @@
       </c>
       <c r="AA21" t="inlineStr">
         <is>
-          <t>/m8ZoSz36OSGjUcbMEAj1ve6WRHq.jpg</t>
+          <t>/1ho0d4LNZw3Y0voeKmSvPSgJOJ2.jpg</t>
         </is>
       </c>
     </row>
@@ -7139,6 +7164,11 @@
           <t>#988d5f</t>
         </is>
       </c>
+      <c r="AA22" t="inlineStr">
+        <is>
+          <t>/bhBKyVeYqyRiGG83d4pdxMKWdaQ.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -7375,6 +7405,11 @@
           <t>#a42823</t>
         </is>
       </c>
+      <c r="AA24" t="inlineStr">
+        <is>
+          <t>/gqgwNjwjSqGkOqkE2rppogenu4v.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -7495,7 +7530,7 @@
       </c>
       <c r="AA25" t="inlineStr">
         <is>
-          <t>/9OPhDJ6kkXZretJgp41h3Pwfnoe.jpg</t>
+          <t>/bj1v6YKF8yHqA489VFfnQvOJpnc.jpg</t>
         </is>
       </c>
     </row>
@@ -7618,7 +7653,7 @@
       </c>
       <c r="AA26" t="inlineStr">
         <is>
-          <t>/qJ2tW6WMUDux911r6m7haRef0WH.jpg</t>
+          <t>/jdvF6UJjtPpaK5HyceiurCrpMGN.jpg</t>
         </is>
       </c>
     </row>
@@ -7741,7 +7776,7 @@
       </c>
       <c r="AA27" t="inlineStr">
         <is>
-          <t>/2GqRAbc6Xcak2ZYrIdTQGbHyTsl.jpg</t>
+          <t>/q6KI8ChlkIYYZww8C053cVfPQRo.jpg</t>
         </is>
       </c>
     </row>
@@ -7864,7 +7899,7 @@
       </c>
       <c r="AA28" t="inlineStr">
         <is>
-          <t>/8uvvuXPINOdKK8gyToq3VNLgDnd.jpg</t>
+          <t>/qbaIViX3tgWSTSFXbldq0ODMdi4.jpg</t>
         </is>
       </c>
     </row>
@@ -7987,7 +8022,7 @@
       </c>
       <c r="AA29" t="inlineStr">
         <is>
-          <t>/xOO4BzaSB4LgAMBVp7FDKiKOxZO.jpg</t>
+          <t>/x2FJsf1ElAgr63Y3PNPtJrcmpoe.jpg</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Use the 28 chosen posters and colours taken from them
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q8auJtZCZpXRhnY2W8Jqqg
</commit_message>
<xml_diff>
--- a/data/films.xlsx
+++ b/data/films.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="사용법" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="추천작" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="제외작" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="사용법" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="추천작" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="제외작" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="229">
+  <fonts count="259">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -936,8 +936,128 @@
       <b val="1"/>
       <color rgb="00d57769"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00ce7e4a"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00f75e51"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00cabba7"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00f16555"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00f46157"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00bb9228"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00eb981f"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00119fc6"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00cbbba8"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001aad94"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="0031a2d2"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="0013a2ad"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00e2e7e1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00b7c2b0"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00f96051"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00c9833f"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00329cce"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00aac3c8"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00bdbebe"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00e9d8c8"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00e56f64"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="008b89db"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00d49548"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00e46d80"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00e6698a"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00eb6a3b"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00f06753"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00cb7f44"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00e46e63"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00f09b28"/>
+    </font>
   </fonts>
-  <fills count="450">
+  <fills count="521">
     <fill>
       <patternFill/>
     </fill>
@@ -3180,6 +3300,361 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="0032221d"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00586d9e"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00b47954"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00162448"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0014161c"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ce1315"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00a9a090"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="006a5d4b"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002d2518"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00383518"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00a51711"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002a2710"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00161d23"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00a90f16"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0027217a"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00bb9228"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00240605"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00eb981f"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00391d1b"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00b7cac1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="006f909d"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00b99c61"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00685a49"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00332401"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="006ea295"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00182a2a"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0057a0c3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002e2b23"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="003c5b5e"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0029261e"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="003b467a"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00e2e7e1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002b261c"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00586252"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0026444f"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ca2c24"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00122a33"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00b38863"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00284f64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00b9d0d2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00849ca1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00172a2c"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="003c3d3d"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0061728a"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00e9d8c8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001b2738"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00f5edb7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00830f11"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002d2701"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00f09b28"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00433d85"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000d0101"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00d3964d"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0033211f"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="003b8bc3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00b44258"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00911644"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002d2425"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00f1edde"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00d95a29"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00e7f0f4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00b2886a"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00010102"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00b22c1c"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00050341"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00192348"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001c1f3e"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0021243e"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00041467"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00231d68"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00202148"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00365384"/>
       </patternFill>
     </fill>
   </fills>
@@ -3195,7 +3670,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="686">
+  <cellXfs count="790">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -3888,6 +4363,110 @@
     <xf numFmtId="0" fontId="228" fillId="449" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="56" fillId="447" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="56" fillId="448" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="230" fillId="216" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="453" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="454" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="457" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="231" fillId="457" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="455" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="456" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="460" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="232" fillId="460" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="458" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="459" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="233" fillId="216" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="461" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="462" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="234" fillId="367" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="463" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="464" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="467" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="235" fillId="467" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="465" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="466" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="452" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="229" fillId="452" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="450" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="451" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="236" fillId="354" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="468" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="469" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="472" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="237" fillId="472" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="470" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="471" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="238" fillId="244" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="473" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="239" fillId="247" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="474" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="475" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="478" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="240" fillId="478" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="476" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="477" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="241" fillId="256" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="479" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="480" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="481" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="242" fillId="481" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="481" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="482" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="485" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="243" fillId="485" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="483" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="484" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="244" fillId="225" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="486" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="245" fillId="247" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="487" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="490" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="246" fillId="490" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="488" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="489" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="247" fillId="273" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="491" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="494" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="248" fillId="494" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="492" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="493" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="497" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="249" fillId="497" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="495" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="496" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="250" fillId="321" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="498" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="499" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="506" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="253" fillId="506" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="505" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="252" fillId="425" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="503" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="504" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="502" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="251" fillId="502" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="500" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="501" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="509" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="510" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="254" fillId="205" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="507" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="508" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="255" fillId="283" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="511" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="512" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="257" fillId="452" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="517" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="519" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="258" fillId="519" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="518" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="514" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="253" fillId="514" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="513" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="516" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="256" fillId="516" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="515" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="254" fillId="318" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="520" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -4789,29 +5368,34 @@
           <t>noir</t>
         </is>
       </c>
-      <c r="W3" s="581" t="inlineStr">
-        <is>
-          <t>#392002</t>
-        </is>
-      </c>
-      <c r="X3" s="582" t="inlineStr">
-        <is>
-          <t>#d47960</t>
-        </is>
-      </c>
-      <c r="Y3" s="583" t="inlineStr">
-        <is>
-          <t>#f99b1a</t>
-        </is>
-      </c>
-      <c r="Z3" s="584" t="inlineStr">
-        <is>
-          <t>#984630</t>
+      <c r="W3" s="324" t="inlineStr">
+        <is>
+          <t>#2d2423</t>
+        </is>
+      </c>
+      <c r="X3" s="686" t="inlineStr">
+        <is>
+          <t>#f75e51</t>
+        </is>
+      </c>
+      <c r="Y3" s="687" t="inlineStr">
+        <is>
+          <t>#14161c</t>
+        </is>
+      </c>
+      <c r="Z3" s="688" t="inlineStr">
+        <is>
+          <t>#ce1315</t>
         </is>
       </c>
       <c r="AA3" t="inlineStr">
         <is>
           <t>/mbm8k3GFhXS0ROd9AD1gqYbIFbM.jpg</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>
@@ -5038,29 +5622,34 @@
           <t>typewriter</t>
         </is>
       </c>
-      <c r="W5" s="482" t="inlineStr">
-        <is>
-          <t>#421610</t>
-        </is>
-      </c>
-      <c r="X5" s="585" t="inlineStr">
-        <is>
-          <t>#6192d9</t>
-        </is>
-      </c>
-      <c r="Y5" s="586" t="inlineStr">
-        <is>
-          <t>#e91d03</t>
-        </is>
-      </c>
-      <c r="Z5" s="587" t="inlineStr">
-        <is>
-          <t>#2a446a</t>
+      <c r="W5" s="689" t="inlineStr">
+        <is>
+          <t>#2d2518</t>
+        </is>
+      </c>
+      <c r="X5" s="690" t="inlineStr">
+        <is>
+          <t>#cabba7</t>
+        </is>
+      </c>
+      <c r="Y5" s="691" t="inlineStr">
+        <is>
+          <t>#a9a090</t>
+        </is>
+      </c>
+      <c r="Z5" s="692" t="inlineStr">
+        <is>
+          <t>#6a5d4b</t>
         </is>
       </c>
       <c r="AA5" t="inlineStr">
         <is>
           <t>/fK4l8KyVZAPlEJ9oUxblz70Qeyy.jpg</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>
@@ -5165,29 +5754,34 @@
           <t>epic</t>
         </is>
       </c>
-      <c r="W6" s="588" t="inlineStr">
-        <is>
-          <t>#2a270c</t>
-        </is>
-      </c>
-      <c r="X6" s="589" t="inlineStr">
-        <is>
-          <t>#9a9530</t>
-        </is>
-      </c>
-      <c r="Y6" s="125" t="inlineStr">
-        <is>
-          <t>#3d3a19</t>
-        </is>
-      </c>
-      <c r="Z6" s="126" t="inlineStr">
-        <is>
-          <t>#888548</t>
+      <c r="W6" s="693" t="inlineStr">
+        <is>
+          <t>#2a2710</t>
+        </is>
+      </c>
+      <c r="X6" s="694" t="inlineStr">
+        <is>
+          <t>#f16555</t>
+        </is>
+      </c>
+      <c r="Y6" s="695" t="inlineStr">
+        <is>
+          <t>#383518</t>
+        </is>
+      </c>
+      <c r="Z6" s="696" t="inlineStr">
+        <is>
+          <t>#a51711</t>
         </is>
       </c>
       <c r="AA6" t="inlineStr">
         <is>
           <t>/4d4mTSfDIFIbUbMLUfaKodvxYXA.jpg</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>
@@ -5293,24 +5887,29 @@
           <t>#2d2423</t>
         </is>
       </c>
-      <c r="X7" s="496" t="inlineStr">
-        <is>
-          <t>#f06462</t>
-        </is>
-      </c>
-      <c r="Y7" s="387" t="inlineStr">
-        <is>
-          <t>#020202</t>
-        </is>
-      </c>
-      <c r="Z7" s="130" t="inlineStr">
-        <is>
-          <t>#b1272e</t>
+      <c r="X7" s="697" t="inlineStr">
+        <is>
+          <t>#f46157</t>
+        </is>
+      </c>
+      <c r="Y7" s="698" t="inlineStr">
+        <is>
+          <t>#161d23</t>
+        </is>
+      </c>
+      <c r="Z7" s="699" t="inlineStr">
+        <is>
+          <t>#a90f16</t>
         </is>
       </c>
       <c r="AA7" t="inlineStr">
         <is>
           <t>/7fn624j5lj3xTme2SgiLCeuedmO.jpg</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>
@@ -5411,29 +6010,34 @@
           <t>script</t>
         </is>
       </c>
-      <c r="W8" s="327" t="inlineStr">
-        <is>
-          <t>#152448</t>
-        </is>
-      </c>
-      <c r="X8" s="497" t="inlineStr">
-        <is>
-          <t>#b38c2b</t>
-        </is>
-      </c>
-      <c r="Y8" s="133" t="inlineStr">
-        <is>
-          <t>#37569d</t>
-        </is>
-      </c>
-      <c r="Z8" s="134" t="inlineStr">
-        <is>
-          <t>#856823</t>
+      <c r="W8" s="557" t="inlineStr">
+        <is>
+          <t>#1f2248</t>
+        </is>
+      </c>
+      <c r="X8" s="700" t="inlineStr">
+        <is>
+          <t>#bb9228</t>
+        </is>
+      </c>
+      <c r="Y8" s="701" t="inlineStr">
+        <is>
+          <t>#27217a</t>
+        </is>
+      </c>
+      <c r="Z8" s="702" t="inlineStr">
+        <is>
+          <t>#bb9228</t>
         </is>
       </c>
       <c r="AA8" t="inlineStr">
         <is>
           <t>/lcYwCSTzCHv0Z2QRpfztt75JyYj.jpg</t>
+        </is>
+      </c>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>
@@ -5534,29 +6138,34 @@
           <t>bold</t>
         </is>
       </c>
-      <c r="W9" s="498" t="inlineStr">
-        <is>
-          <t>#401a01</t>
-        </is>
-      </c>
-      <c r="X9" s="499" t="inlineStr">
-        <is>
-          <t>#e1b65b</t>
-        </is>
-      </c>
-      <c r="Y9" s="137" t="inlineStr">
-        <is>
-          <t>#db6c21</t>
-        </is>
-      </c>
-      <c r="Z9" s="500" t="inlineStr">
-        <is>
-          <t>#deb767</t>
+      <c r="W9" s="703" t="inlineStr">
+        <is>
+          <t>#391d1b</t>
+        </is>
+      </c>
+      <c r="X9" s="704" t="inlineStr">
+        <is>
+          <t>#eb981f</t>
+        </is>
+      </c>
+      <c r="Y9" s="705" t="inlineStr">
+        <is>
+          <t>#240605</t>
+        </is>
+      </c>
+      <c r="Z9" s="706" t="inlineStr">
+        <is>
+          <t>#eb981f</t>
         </is>
       </c>
       <c r="AA9" t="inlineStr">
         <is>
           <t>/jtTHxuJhuZpFAnCI4vGjg1LGmpY.jpg</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>
@@ -5657,24 +6266,24 @@
           <t>mono</t>
         </is>
       </c>
-      <c r="W10" s="433" t="inlineStr">
-        <is>
-          <t>#182448</t>
-        </is>
-      </c>
-      <c r="X10" s="678" t="inlineStr">
-        <is>
-          <t>#d9994d</t>
-        </is>
-      </c>
-      <c r="Y10" s="593" t="inlineStr">
-        <is>
-          <t>#4c62a4</t>
-        </is>
-      </c>
-      <c r="Z10" s="592" t="inlineStr">
-        <is>
-          <t>#c1a280</t>
+      <c r="W10" s="707" t="inlineStr">
+        <is>
+          <t>#162448</t>
+        </is>
+      </c>
+      <c r="X10" s="708" t="inlineStr">
+        <is>
+          <t>#ce7e4a</t>
+        </is>
+      </c>
+      <c r="Y10" s="709" t="inlineStr">
+        <is>
+          <t>#586d9e</t>
+        </is>
+      </c>
+      <c r="Z10" s="710" t="inlineStr">
+        <is>
+          <t>#b47954</t>
         </is>
       </c>
       <c r="AA10" t="inlineStr">
@@ -5685,6 +6294,11 @@
       <c r="AB10" t="inlineStr">
         <is>
           <t>파랑</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>
@@ -6161,29 +6775,34 @@
           <t>bold</t>
         </is>
       </c>
-      <c r="W14" s="369" t="inlineStr">
-        <is>
-          <t>#2b251f</t>
-        </is>
-      </c>
-      <c r="X14" s="602" t="inlineStr">
-        <is>
-          <t>#e68f2c</t>
-        </is>
-      </c>
-      <c r="Y14" s="603" t="inlineStr">
-        <is>
-          <t>#cae2e2</t>
-        </is>
-      </c>
-      <c r="Z14" s="604" t="inlineStr">
-        <is>
-          <t>#e68f2c</t>
+      <c r="W14" s="532" t="inlineStr">
+        <is>
+          <t>#1f282c</t>
+        </is>
+      </c>
+      <c r="X14" s="711" t="inlineStr">
+        <is>
+          <t>#119fc6</t>
+        </is>
+      </c>
+      <c r="Y14" s="712" t="inlineStr">
+        <is>
+          <t>#b7cac1</t>
+        </is>
+      </c>
+      <c r="Z14" s="713" t="inlineStr">
+        <is>
+          <t>#6f909d</t>
         </is>
       </c>
       <c r="AA14" t="inlineStr">
         <is>
           <t>/2e853FDVSIso600RqAMunPxiZjq.jpg</t>
+        </is>
+      </c>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>
@@ -6402,29 +7021,34 @@
           <t>bold</t>
         </is>
       </c>
-      <c r="W16" s="335" t="inlineStr">
-        <is>
-          <t>#2c2520</t>
-        </is>
-      </c>
-      <c r="X16" s="605" t="inlineStr">
-        <is>
-          <t>#ce8048</t>
-        </is>
-      </c>
-      <c r="Y16" s="166" t="inlineStr">
-        <is>
-          <t>#040308</t>
-        </is>
-      </c>
-      <c r="Z16" s="165" t="inlineStr">
-        <is>
-          <t>#a87756</t>
+      <c r="W16" s="714" t="inlineStr">
+        <is>
+          <t>#332401</t>
+        </is>
+      </c>
+      <c r="X16" s="715" t="inlineStr">
+        <is>
+          <t>#cbbba8</t>
+        </is>
+      </c>
+      <c r="Y16" s="716" t="inlineStr">
+        <is>
+          <t>#b99c61</t>
+        </is>
+      </c>
+      <c r="Z16" s="717" t="inlineStr">
+        <is>
+          <t>#685a49</t>
         </is>
       </c>
       <c r="AA16" t="inlineStr">
         <is>
           <t>/f6ORXXQdIKHU3RvC6AC2lwAD6Mq.jpg</t>
+        </is>
+      </c>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>
@@ -6525,29 +7149,34 @@
           <t>typewriter</t>
         </is>
       </c>
-      <c r="W17" s="482" t="inlineStr">
-        <is>
-          <t>#421610</t>
-        </is>
-      </c>
-      <c r="X17" s="606" t="inlineStr">
-        <is>
-          <t>#ead373</t>
-        </is>
-      </c>
-      <c r="Y17" s="607" t="inlineStr">
-        <is>
-          <t>#b13b2c</t>
-        </is>
-      </c>
-      <c r="Z17" s="608" t="inlineStr">
-        <is>
-          <t>#e4d490</t>
+      <c r="W17" s="361" t="inlineStr">
+        <is>
+          <t>#1f2926</t>
+        </is>
+      </c>
+      <c r="X17" s="718" t="inlineStr">
+        <is>
+          <t>#1aad94</t>
+        </is>
+      </c>
+      <c r="Y17" s="363" t="inlineStr">
+        <is>
+          <t>#060606</t>
+        </is>
+      </c>
+      <c r="Z17" s="719" t="inlineStr">
+        <is>
+          <t>#6ea295</t>
         </is>
       </c>
       <c r="AA17" t="inlineStr">
         <is>
           <t>/cVUDMnskSc01rdbyH0tLATTJUdP.jpg</t>
+        </is>
+      </c>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>
@@ -6648,29 +7277,34 @@
           <t>gothic</t>
         </is>
       </c>
-      <c r="W18" s="324" t="inlineStr">
-        <is>
-          <t>#2d2423</t>
-        </is>
-      </c>
-      <c r="X18" s="609" t="inlineStr">
-        <is>
-          <t>#f0655c</t>
-        </is>
-      </c>
-      <c r="Y18" s="610" t="inlineStr">
-        <is>
-          <t>#030302</t>
-        </is>
-      </c>
-      <c r="Z18" s="611" t="inlineStr">
-        <is>
-          <t>#a11419</t>
+      <c r="W18" s="365" t="inlineStr">
+        <is>
+          <t>#20282c</t>
+        </is>
+      </c>
+      <c r="X18" s="720" t="inlineStr">
+        <is>
+          <t>#31a2d2</t>
+        </is>
+      </c>
+      <c r="Y18" s="721" t="inlineStr">
+        <is>
+          <t>#182a2a</t>
+        </is>
+      </c>
+      <c r="Z18" s="722" t="inlineStr">
+        <is>
+          <t>#57a0c3</t>
         </is>
       </c>
       <c r="AA18" t="inlineStr">
         <is>
           <t>/s8C4whhKtDaJvMDcyiMvx3BIF5F.jpg</t>
+        </is>
+      </c>
+      <c r="AC18" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>
@@ -6771,29 +7405,34 @@
           <t>elegant</t>
         </is>
       </c>
-      <c r="W19" s="612" t="inlineStr">
-        <is>
-          <t>#0b2c2d</t>
-        </is>
-      </c>
-      <c r="X19" s="613" t="inlineStr">
-        <is>
-          <t>#c28736</t>
-        </is>
-      </c>
-      <c r="Y19" s="614" t="inlineStr">
-        <is>
-          <t>#345b5c</t>
-        </is>
-      </c>
-      <c r="Z19" s="615" t="inlineStr">
-        <is>
-          <t>#a08769</t>
+      <c r="W19" s="723" t="inlineStr">
+        <is>
+          <t>#29261e</t>
+        </is>
+      </c>
+      <c r="X19" s="724" t="inlineStr">
+        <is>
+          <t>#13a2ad</t>
+        </is>
+      </c>
+      <c r="Y19" s="725" t="inlineStr">
+        <is>
+          <t>#2e2b23</t>
+        </is>
+      </c>
+      <c r="Z19" s="726" t="inlineStr">
+        <is>
+          <t>#3c5b5e</t>
         </is>
       </c>
       <c r="AA19" t="inlineStr">
         <is>
           <t>/11zlNdxiHhhW5BWgL2PkqaRCzTM.jpg</t>
+        </is>
+      </c>
+      <c r="AC19" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>
@@ -7017,29 +7656,34 @@
           <t>classic</t>
         </is>
       </c>
-      <c r="W21" s="620" t="inlineStr">
-        <is>
-          <t>#1f2635</t>
-        </is>
-      </c>
-      <c r="X21" s="621" t="inlineStr">
-        <is>
-          <t>#dd707e</t>
-        </is>
-      </c>
-      <c r="Y21" s="622" t="inlineStr">
-        <is>
-          <t>#161e2f</t>
-        </is>
-      </c>
-      <c r="Z21" s="623" t="inlineStr">
-        <is>
-          <t>#942e41</t>
+      <c r="W21" s="377" t="inlineStr">
+        <is>
+          <t>#1c2348</t>
+        </is>
+      </c>
+      <c r="X21" s="727" t="inlineStr">
+        <is>
+          <t>#e2e7e1</t>
+        </is>
+      </c>
+      <c r="Y21" s="728" t="inlineStr">
+        <is>
+          <t>#3b467a</t>
+        </is>
+      </c>
+      <c r="Z21" s="729" t="inlineStr">
+        <is>
+          <t>#e2e7e1</t>
         </is>
       </c>
       <c r="AA21" t="inlineStr">
         <is>
           <t>/1ho0d4LNZw3Y0voeKmSvPSgJOJ2.jpg</t>
+        </is>
+      </c>
+      <c r="AC21" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>
@@ -7144,29 +7788,34 @@
           <t>gothic</t>
         </is>
       </c>
-      <c r="W22" s="381" t="inlineStr">
-        <is>
-          <t>#28271f</t>
-        </is>
-      </c>
-      <c r="X22" s="526" t="inlineStr">
-        <is>
-          <t>#a7912a</t>
-        </is>
-      </c>
-      <c r="Y22" s="189" t="inlineStr">
-        <is>
-          <t>#211010</t>
-        </is>
-      </c>
-      <c r="Z22" s="190" t="inlineStr">
-        <is>
-          <t>#988d5f</t>
+      <c r="W22" s="730" t="inlineStr">
+        <is>
+          <t>#2b261c</t>
+        </is>
+      </c>
+      <c r="X22" s="731" t="inlineStr">
+        <is>
+          <t>#b7c2b0</t>
+        </is>
+      </c>
+      <c r="Y22" s="732" t="inlineStr">
+        <is>
+          <t>#2b261c</t>
+        </is>
+      </c>
+      <c r="Z22" s="733" t="inlineStr">
+        <is>
+          <t>#586252</t>
         </is>
       </c>
       <c r="AA22" t="inlineStr">
         <is>
           <t>/bhBKyVeYqyRiGG83d4pdxMKWdaQ.jpg</t>
+        </is>
+      </c>
+      <c r="AC22" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>
@@ -7385,29 +8034,34 @@
           <t>scifi</t>
         </is>
       </c>
-      <c r="W24" s="529" t="inlineStr">
-        <is>
-          <t>#022b39</t>
-        </is>
-      </c>
-      <c r="X24" s="530" t="inlineStr">
-        <is>
-          <t>#eb6b5f</t>
-        </is>
-      </c>
-      <c r="Y24" s="197" t="inlineStr">
-        <is>
-          <t>#2c647a</t>
-        </is>
-      </c>
-      <c r="Z24" s="198" t="inlineStr">
-        <is>
-          <t>#a42823</t>
+      <c r="W24" s="734" t="inlineStr">
+        <is>
+          <t>#122a33</t>
+        </is>
+      </c>
+      <c r="X24" s="735" t="inlineStr">
+        <is>
+          <t>#f96051</t>
+        </is>
+      </c>
+      <c r="Y24" s="736" t="inlineStr">
+        <is>
+          <t>#26444f</t>
+        </is>
+      </c>
+      <c r="Z24" s="737" t="inlineStr">
+        <is>
+          <t>#ca2c24</t>
         </is>
       </c>
       <c r="AA24" t="inlineStr">
         <is>
           <t>/gqgwNjwjSqGkOqkE2rppogenu4v.jpg</t>
+        </is>
+      </c>
+      <c r="AC24" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>
@@ -7508,29 +8162,34 @@
           <t>western</t>
         </is>
       </c>
-      <c r="W25" s="468" t="inlineStr">
-        <is>
-          <t>#392001</t>
-        </is>
-      </c>
-      <c r="X25" s="624" t="inlineStr">
-        <is>
-          <t>#d67681</t>
-        </is>
-      </c>
-      <c r="Y25" s="625" t="inlineStr">
-        <is>
-          <t>#eaa34f</t>
-        </is>
-      </c>
-      <c r="Z25" s="626" t="inlineStr">
-        <is>
-          <t>#573236</t>
+      <c r="W25" s="335" t="inlineStr">
+        <is>
+          <t>#2c2520</t>
+        </is>
+      </c>
+      <c r="X25" s="738" t="inlineStr">
+        <is>
+          <t>#c9833f</t>
+        </is>
+      </c>
+      <c r="Y25" s="337" t="inlineStr">
+        <is>
+          <t>#020101</t>
+        </is>
+      </c>
+      <c r="Z25" s="739" t="inlineStr">
+        <is>
+          <t>#b38863</t>
         </is>
       </c>
       <c r="AA25" t="inlineStr">
         <is>
           <t>/bj1v6YKF8yHqA489VFfnQvOJpnc.jpg</t>
+        </is>
+      </c>
+      <c r="AC25" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>
@@ -7631,29 +8290,34 @@
           <t>bold</t>
         </is>
       </c>
-      <c r="W26" s="627" t="inlineStr">
-        <is>
-          <t>#172839</t>
-        </is>
-      </c>
-      <c r="X26" s="679" t="inlineStr">
-        <is>
-          <t>#ee694f</t>
-        </is>
-      </c>
-      <c r="Y26" s="629" t="inlineStr">
-        <is>
-          <t>#0d2135</t>
-        </is>
-      </c>
-      <c r="Z26" s="680" t="inlineStr">
-        <is>
-          <t>#b9381f</t>
+      <c r="W26" s="365" t="inlineStr">
+        <is>
+          <t>#20282c</t>
+        </is>
+      </c>
+      <c r="X26" s="740" t="inlineStr">
+        <is>
+          <t>#329cce</t>
+        </is>
+      </c>
+      <c r="Y26" s="205" t="inlineStr">
+        <is>
+          <t>#000001</t>
+        </is>
+      </c>
+      <c r="Z26" s="741" t="inlineStr">
+        <is>
+          <t>#284f64</t>
         </is>
       </c>
       <c r="AA26" t="inlineStr">
         <is>
           <t>/jdvF6UJjtPpaK5HyceiurCrpMGN.jpg</t>
+        </is>
+      </c>
+      <c r="AC26" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>
@@ -7754,29 +8418,34 @@
           <t>scifi</t>
         </is>
       </c>
-      <c r="W27" s="631" t="inlineStr">
-        <is>
-          <t>#092746</t>
-        </is>
-      </c>
-      <c r="X27" s="632" t="inlineStr">
-        <is>
-          <t>#cf8049</t>
-        </is>
-      </c>
-      <c r="Y27" s="633" t="inlineStr">
-        <is>
-          <t>#4d739e</t>
-        </is>
-      </c>
-      <c r="Z27" s="634" t="inlineStr">
-        <is>
-          <t>#c4865c</t>
+      <c r="W27" s="742" t="inlineStr">
+        <is>
+          <t>#172a2c</t>
+        </is>
+      </c>
+      <c r="X27" s="743" t="inlineStr">
+        <is>
+          <t>#aac3c8</t>
+        </is>
+      </c>
+      <c r="Y27" s="744" t="inlineStr">
+        <is>
+          <t>#b9d0d2</t>
+        </is>
+      </c>
+      <c r="Z27" s="745" t="inlineStr">
+        <is>
+          <t>#849ca1</t>
         </is>
       </c>
       <c r="AA27" t="inlineStr">
         <is>
           <t>/q6KI8ChlkIYYZww8C053cVfPQRo.jpg</t>
+        </is>
+      </c>
+      <c r="AC27" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>
@@ -7877,29 +8546,34 @@
           <t>noir</t>
         </is>
       </c>
-      <c r="W28" s="635" t="inlineStr">
-        <is>
-          <t>#21272d</t>
-        </is>
-      </c>
-      <c r="X28" s="636" t="inlineStr">
-        <is>
-          <t>#4498d4</t>
-        </is>
-      </c>
-      <c r="Y28" s="637" t="inlineStr">
-        <is>
-          <t>#192022</t>
-        </is>
-      </c>
-      <c r="Z28" s="638" t="inlineStr">
-        <is>
-          <t>#346d96</t>
+      <c r="W28" s="402" t="inlineStr">
+        <is>
+          <t>#262626</t>
+        </is>
+      </c>
+      <c r="X28" s="746" t="inlineStr">
+        <is>
+          <t>#bdbebe</t>
+        </is>
+      </c>
+      <c r="Y28" s="535" t="inlineStr">
+        <is>
+          <t>#fefefe</t>
+        </is>
+      </c>
+      <c r="Z28" s="747" t="inlineStr">
+        <is>
+          <t>#3c3d3d</t>
         </is>
       </c>
       <c r="AA28" t="inlineStr">
         <is>
           <t>/qbaIViX3tgWSTSFXbldq0ODMdi4.jpg</t>
+        </is>
+      </c>
+      <c r="AC28" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>
@@ -8000,29 +8674,34 @@
           <t>light</t>
         </is>
       </c>
-      <c r="W29" s="639" t="inlineStr">
-        <is>
-          <t>#342209</t>
-        </is>
-      </c>
-      <c r="X29" s="640" t="inlineStr">
-        <is>
-          <t>#d17c53</t>
-        </is>
-      </c>
-      <c r="Y29" s="641" t="inlineStr">
-        <is>
-          <t>#e2c6a4</t>
-        </is>
-      </c>
-      <c r="Z29" s="642" t="inlineStr">
-        <is>
-          <t>#a26f57</t>
+      <c r="W29" s="748" t="inlineStr">
+        <is>
+          <t>#1b2738</t>
+        </is>
+      </c>
+      <c r="X29" s="749" t="inlineStr">
+        <is>
+          <t>#e9d8c8</t>
+        </is>
+      </c>
+      <c r="Y29" s="750" t="inlineStr">
+        <is>
+          <t>#61728a</t>
+        </is>
+      </c>
+      <c r="Z29" s="751" t="inlineStr">
+        <is>
+          <t>#e9d8c8</t>
         </is>
       </c>
       <c r="AA29" t="inlineStr">
         <is>
           <t>/x2FJsf1ElAgr63Y3PNPtJrcmpoe.jpg</t>
+        </is>
+      </c>
+      <c r="AC29" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>
@@ -8849,29 +9528,39 @@
           <t>comic</t>
         </is>
       </c>
-      <c r="W36" s="550" t="inlineStr">
-        <is>
-          <t>#3f1529</t>
-        </is>
-      </c>
-      <c r="X36" s="551" t="inlineStr">
-        <is>
-          <t>#648de6</t>
-        </is>
-      </c>
-      <c r="Y36" s="245" t="inlineStr">
-        <is>
-          <t>#f2439d</t>
-        </is>
-      </c>
-      <c r="Z36" s="246" t="inlineStr">
-        <is>
-          <t>#4a71c7</t>
+      <c r="W36" s="707" t="inlineStr">
+        <is>
+          <t>#162448</t>
+        </is>
+      </c>
+      <c r="X36" s="777" t="inlineStr">
+        <is>
+          <t>#e46e63</t>
+        </is>
+      </c>
+      <c r="Y36" s="778" t="inlineStr">
+        <is>
+          <t>#041467</t>
+        </is>
+      </c>
+      <c r="Z36" s="755" t="inlineStr">
+        <is>
+          <t>#830f11</t>
         </is>
       </c>
       <c r="AA36" t="inlineStr">
         <is>
           <t>/aCXPF21O3jM1mCT1iFVYDNmsWIe.jpg</t>
+        </is>
+      </c>
+      <c r="AB36" t="inlineStr">
+        <is>
+          <t>파랑</t>
+        </is>
+      </c>
+      <c r="AC36" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>
@@ -8972,29 +9661,39 @@
           <t>script</t>
         </is>
       </c>
-      <c r="W37" s="552" t="inlineStr">
-        <is>
-          <t>#391d21</t>
-        </is>
-      </c>
-      <c r="X37" s="553" t="inlineStr">
-        <is>
-          <t>#5e92d9</t>
-        </is>
-      </c>
-      <c r="Y37" s="554" t="inlineStr">
-        <is>
-          <t>#532f34</t>
-        </is>
-      </c>
-      <c r="Z37" s="555" t="inlineStr">
-        <is>
-          <t>#5078ae</t>
+      <c r="W37" s="779" t="inlineStr">
+        <is>
+          <t>#202148</t>
+        </is>
+      </c>
+      <c r="X37" s="780" t="inlineStr">
+        <is>
+          <t>#f09b28</t>
+        </is>
+      </c>
+      <c r="Y37" s="781" t="inlineStr">
+        <is>
+          <t>#231d68</t>
+        </is>
+      </c>
+      <c r="Z37" s="757" t="inlineStr">
+        <is>
+          <t>#f09b28</t>
         </is>
       </c>
       <c r="AA37" t="inlineStr">
         <is>
           <t>/48mdKcYKIVfRtoSCqhkY8xMzJlA.jpg</t>
+        </is>
+      </c>
+      <c r="AB37" t="inlineStr">
+        <is>
+          <t>보라</t>
+        </is>
+      </c>
+      <c r="AC37" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>
@@ -9095,29 +9794,39 @@
           <t>hand</t>
         </is>
       </c>
-      <c r="W38" s="436" t="inlineStr">
-        <is>
-          <t>#212147</t>
-        </is>
-      </c>
-      <c r="X38" s="556" t="inlineStr">
-        <is>
-          <t>#63a64b</t>
-        </is>
-      </c>
-      <c r="Y38" s="253" t="inlineStr">
-        <is>
-          <t>#1d194d</t>
-        </is>
-      </c>
-      <c r="Z38" s="254" t="inlineStr">
-        <is>
-          <t>#63a64b</t>
+      <c r="W38" s="782" t="inlineStr">
+        <is>
+          <t>#192348</t>
+        </is>
+      </c>
+      <c r="X38" s="783" t="inlineStr">
+        <is>
+          <t>#e6698a</t>
+        </is>
+      </c>
+      <c r="Y38" s="784" t="inlineStr">
+        <is>
+          <t>#050341</t>
+        </is>
+      </c>
+      <c r="Z38" s="761" t="inlineStr">
+        <is>
+          <t>#911644</t>
         </is>
       </c>
       <c r="AA38" t="inlineStr">
         <is>
           <t>/lRHE0vzf3oYJrhbsHXjIkF4Tl5A.jpg</t>
+        </is>
+      </c>
+      <c r="AB38" t="inlineStr">
+        <is>
+          <t>남색</t>
+        </is>
+      </c>
+      <c r="AC38" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>
@@ -9454,29 +10163,34 @@
           <t>retro</t>
         </is>
       </c>
-      <c r="W41" s="448" t="inlineStr">
-        <is>
-          <t>#022a3f</t>
-        </is>
-      </c>
-      <c r="X41" s="561" t="inlineStr">
-        <is>
-          <t>#d57687</t>
-        </is>
-      </c>
-      <c r="Y41" s="265" t="inlineStr">
-        <is>
-          <t>#2496d3</t>
-        </is>
-      </c>
-      <c r="Z41" s="266" t="inlineStr">
-        <is>
-          <t>#af6874</t>
+      <c r="W41" s="647" t="inlineStr">
+        <is>
+          <t>#022942</t>
+        </is>
+      </c>
+      <c r="X41" s="762" t="inlineStr">
+        <is>
+          <t>#e46d80</t>
+        </is>
+      </c>
+      <c r="Y41" s="763" t="inlineStr">
+        <is>
+          <t>#3b8bc3</t>
+        </is>
+      </c>
+      <c r="Z41" s="764" t="inlineStr">
+        <is>
+          <t>#b44258</t>
         </is>
       </c>
       <c r="AA41" t="inlineStr">
         <is>
           <t>/nlV35BhheFq9QqIdiL8aMCa3zAm.jpg</t>
+        </is>
+      </c>
+      <c r="AC41" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>
@@ -9695,29 +10409,34 @@
           <t>typewriter</t>
         </is>
       </c>
-      <c r="W43" s="662" t="inlineStr">
-        <is>
-          <t>#072747</t>
-        </is>
-      </c>
-      <c r="X43" s="663" t="inlineStr">
-        <is>
-          <t>#db8064</t>
-        </is>
-      </c>
-      <c r="Y43" s="664" t="inlineStr">
-        <is>
-          <t>#5985b6</t>
-        </is>
-      </c>
-      <c r="Z43" s="665" t="inlineStr">
-        <is>
-          <t>#d0866f</t>
+      <c r="W43" s="765" t="inlineStr">
+        <is>
+          <t>#33211f</t>
+        </is>
+      </c>
+      <c r="X43" s="766" t="inlineStr">
+        <is>
+          <t>#d49548</t>
+        </is>
+      </c>
+      <c r="Y43" s="767" t="inlineStr">
+        <is>
+          <t>#0d0101</t>
+        </is>
+      </c>
+      <c r="Z43" s="768" t="inlineStr">
+        <is>
+          <t>#d3964d</t>
         </is>
       </c>
       <c r="AA43" t="inlineStr">
         <is>
           <t>/9cqNxx0GxF0bflZmeSMuL5tnGzr.jpg</t>
+        </is>
+      </c>
+      <c r="AC43" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>
@@ -9936,29 +10655,39 @@
           <t>elegant</t>
         </is>
       </c>
-      <c r="W45" s="666" t="inlineStr">
-        <is>
-          <t>#162931</t>
-        </is>
-      </c>
-      <c r="X45" s="667" t="inlineStr">
-        <is>
-          <t>#c8893c</t>
-        </is>
-      </c>
-      <c r="Y45" s="668" t="inlineStr">
-        <is>
-          <t>#c9e5f1</t>
-        </is>
-      </c>
-      <c r="Z45" s="669" t="inlineStr">
-        <is>
-          <t>#af9273</t>
+      <c r="W45" s="785" t="inlineStr">
+        <is>
+          <t>#21243e</t>
+        </is>
+      </c>
+      <c r="X45" s="786" t="inlineStr">
+        <is>
+          <t>#cb7f44</t>
+        </is>
+      </c>
+      <c r="Y45" s="787" t="inlineStr">
+        <is>
+          <t>#1c1f3e</t>
+        </is>
+      </c>
+      <c r="Z45" s="770" t="inlineStr">
+        <is>
+          <t>#b2886a</t>
         </is>
       </c>
       <c r="AA45" t="inlineStr">
         <is>
           <t>/tKXgTQSwASOXwjlsToWaqDbAJwp.jpg</t>
+        </is>
+      </c>
+      <c r="AB45" t="inlineStr">
+        <is>
+          <t>남색</t>
+        </is>
+      </c>
+      <c r="AC45" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>
@@ -10064,24 +10793,34 @@
           <t>#112548</t>
         </is>
       </c>
-      <c r="X46" s="681" t="inlineStr">
-        <is>
-          <t>#eac262</t>
-        </is>
-      </c>
-      <c r="Y46" s="284" t="inlineStr">
-        <is>
-          <t>#04255b</t>
-        </is>
-      </c>
-      <c r="Z46" s="285" t="inlineStr">
-        <is>
-          <t>#eac262</t>
+      <c r="X46" s="788" t="inlineStr">
+        <is>
+          <t>#eb6a3b</t>
+        </is>
+      </c>
+      <c r="Y46" s="789" t="inlineStr">
+        <is>
+          <t>#365384</t>
+        </is>
+      </c>
+      <c r="Z46" s="773" t="inlineStr">
+        <is>
+          <t>#d95a29</t>
         </is>
       </c>
       <c r="AA46" t="inlineStr">
         <is>
           <t>/7fT4fQtDbueYtWv7NLBHnemSwNF.jpg</t>
+        </is>
+      </c>
+      <c r="AB46" t="inlineStr">
+        <is>
+          <t>남색</t>
+        </is>
+      </c>
+      <c r="AC46" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>
@@ -10300,29 +11039,34 @@
           <t>bold</t>
         </is>
       </c>
-      <c r="W48" s="674" t="inlineStr">
-        <is>
-          <t>#421611</t>
-        </is>
-      </c>
-      <c r="X48" s="675" t="inlineStr">
-        <is>
-          <t>#f7e91e</t>
-        </is>
-      </c>
-      <c r="Y48" s="676" t="inlineStr">
-        <is>
-          <t>#e83b2d</t>
-        </is>
-      </c>
-      <c r="Z48" s="677" t="inlineStr">
-        <is>
-          <t>#f7e909</t>
+      <c r="W48" s="416" t="inlineStr">
+        <is>
+          <t>#2d2422</t>
+        </is>
+      </c>
+      <c r="X48" s="774" t="inlineStr">
+        <is>
+          <t>#f06753</t>
+        </is>
+      </c>
+      <c r="Y48" s="775" t="inlineStr">
+        <is>
+          <t>#010102</t>
+        </is>
+      </c>
+      <c r="Z48" s="776" t="inlineStr">
+        <is>
+          <t>#b22c1c</t>
         </is>
       </c>
       <c r="AA48" t="inlineStr">
         <is>
           <t>/yae986V8wJsh2bPJkYfQ5kmLSw6.jpg</t>
+        </is>
+      </c>
+      <c r="AC48" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
The Irishman: dark blue base, red point from the poster
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q8auJtZCZpXRhnY2W8Jqqg
</commit_message>
<xml_diff>
--- a/data/films.xlsx
+++ b/data/films.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="259">
+  <fonts count="260">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -1056,8 +1056,12 @@
       <b val="1"/>
       <color rgb="00f09b28"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00f75f4f"/>
+    </font>
   </fonts>
-  <fills count="521">
+  <fills count="524">
     <fill>
       <patternFill/>
     </fill>
@@ -3655,6 +3659,21 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00365384"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="003d5263"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00e20b0c"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00182835"/>
       </patternFill>
     </fill>
   </fills>
@@ -3670,7 +3689,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="790">
+  <cellXfs count="794">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -4467,6 +4486,10 @@
     <xf numFmtId="0" fontId="56" fillId="515" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="254" fillId="318" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="56" fillId="520" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="523" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="259" fillId="523" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="521" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="522" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -5368,29 +5391,34 @@
           <t>noir</t>
         </is>
       </c>
-      <c r="W3" s="324" t="inlineStr">
-        <is>
-          <t>#2d2423</t>
-        </is>
-      </c>
-      <c r="X3" s="686" t="inlineStr">
-        <is>
-          <t>#f75e51</t>
-        </is>
-      </c>
-      <c r="Y3" s="687" t="inlineStr">
-        <is>
-          <t>#14161c</t>
-        </is>
-      </c>
-      <c r="Z3" s="688" t="inlineStr">
-        <is>
-          <t>#ce1315</t>
+      <c r="W3" s="790" t="inlineStr">
+        <is>
+          <t>#182835</t>
+        </is>
+      </c>
+      <c r="X3" s="791" t="inlineStr">
+        <is>
+          <t>#f75f4f</t>
+        </is>
+      </c>
+      <c r="Y3" s="792" t="inlineStr">
+        <is>
+          <t>#3d5263</t>
+        </is>
+      </c>
+      <c r="Z3" s="793" t="inlineStr">
+        <is>
+          <t>#e20b0c</t>
         </is>
       </c>
       <c r="AA3" t="inlineStr">
         <is>
           <t>/mbm8k3GFhXS0ROd9AD1gqYbIFbM.jpg</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>남색</t>
         </is>
       </c>
       <c r="AC3" t="inlineStr">

</xml_diff>

<commit_message>
Arcade banner for The Two Popes; Whiplash charcoal base with red point
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q8auJtZCZpXRhnY2W8Jqqg
</commit_message>
<xml_diff>
--- a/data/films.xlsx
+++ b/data/films.xlsx
@@ -1061,7 +1061,7 @@
       <color rgb="00f75f4f"/>
     </font>
   </fonts>
-  <fills count="524">
+  <fills count="525">
     <fill>
       <patternFill/>
     </fill>
@@ -3674,6 +3674,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00182835"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00242629"/>
       </patternFill>
     </fill>
   </fills>
@@ -3689,7 +3694,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="794">
+  <cellXfs count="796">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -4490,6 +4495,8 @@
     <xf numFmtId="0" fontId="259" fillId="523" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="56" fillId="521" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="56" fillId="522" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="524" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="233" fillId="524" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -5774,7 +5781,7 @@
       </c>
       <c r="U6" s="3" t="inlineStr">
         <is>
-          <t>arch</t>
+          <t>arcade</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
@@ -5910,12 +5917,12 @@
           <t>bold</t>
         </is>
       </c>
-      <c r="W7" s="324" t="inlineStr">
-        <is>
-          <t>#2d2423</t>
-        </is>
-      </c>
-      <c r="X7" s="697" t="inlineStr">
+      <c r="W7" s="794" t="inlineStr">
+        <is>
+          <t>#242629</t>
+        </is>
+      </c>
+      <c r="X7" s="795" t="inlineStr">
         <is>
           <t>#f46157</t>
         </is>
@@ -11461,7 +11468,7 @@
       <formula1>"O"</formula1>
     </dataValidation>
     <dataValidation sqref="U2:U500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"sun,waves,bands,rings,split,peaks,arch,rays,grid,dots,trees"</formula1>
+      <formula1>"arcade,sun,waves,bands,rings,split,peaks,arch,rays,grid,dots,trees"</formula1>
     </dataValidation>
     <dataValidation sqref="V2:V500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"classic,elegant,noir,epic,typewriter,mono,bold,scifi,gothic,western,retro,script,hand,comic,light,neon"</formula1>

</xml_diff>

<commit_message>
Banner colours stay in their own hues; Oppenheimer orange/yellow, Spotlight blue-grey/red
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q8auJtZCZpXRhnY2W8Jqqg
</commit_message>
<xml_diff>
--- a/data/films.xlsx
+++ b/data/films.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="260">
+  <fonts count="262">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -1060,8 +1060,16 @@
       <b val="1"/>
       <color rgb="00f75f4f"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00f9d548"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00ff786f"/>
+    </font>
   </fonts>
-  <fills count="525">
+  <fills count="531">
     <fill>
       <patternFill/>
     </fill>
@@ -3679,6 +3687,36 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00242629"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00d76314"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00f9d548"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00582403"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="005c6c80"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00c8262a"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00283546"/>
       </patternFill>
     </fill>
   </fills>
@@ -3694,7 +3732,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="796">
+  <cellXfs count="804">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -4497,6 +4535,14 @@
     <xf numFmtId="0" fontId="56" fillId="522" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="524" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="233" fillId="524" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="527" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="260" fillId="527" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="525" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="526" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="530" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="261" fillId="530" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="528" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="529" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -6173,24 +6219,24 @@
           <t>bold</t>
         </is>
       </c>
-      <c r="W9" s="703" t="inlineStr">
-        <is>
-          <t>#391d1b</t>
-        </is>
-      </c>
-      <c r="X9" s="704" t="inlineStr">
-        <is>
-          <t>#eb981f</t>
-        </is>
-      </c>
-      <c r="Y9" s="705" t="inlineStr">
-        <is>
-          <t>#240605</t>
-        </is>
-      </c>
-      <c r="Z9" s="706" t="inlineStr">
-        <is>
-          <t>#eb981f</t>
+      <c r="W9" s="796" t="inlineStr">
+        <is>
+          <t>#582403</t>
+        </is>
+      </c>
+      <c r="X9" s="797" t="inlineStr">
+        <is>
+          <t>#f9d548</t>
+        </is>
+      </c>
+      <c r="Y9" s="798" t="inlineStr">
+        <is>
+          <t>#d76314</t>
+        </is>
+      </c>
+      <c r="Z9" s="799" t="inlineStr">
+        <is>
+          <t>#f9d548</t>
         </is>
       </c>
       <c r="AA9" t="inlineStr">
@@ -6434,29 +6480,34 @@
           <t>typewriter</t>
         </is>
       </c>
-      <c r="W11" s="324" t="inlineStr">
-        <is>
-          <t>#2d2423</t>
-        </is>
-      </c>
-      <c r="X11" s="594" t="inlineStr">
-        <is>
-          <t>#ef6660</t>
-        </is>
-      </c>
-      <c r="Y11" s="595" t="inlineStr">
-        <is>
-          <t>#e4e4e7</t>
-        </is>
-      </c>
-      <c r="Z11" s="596" t="inlineStr">
-        <is>
-          <t>#b83233</t>
+      <c r="W11" s="800" t="inlineStr">
+        <is>
+          <t>#283546</t>
+        </is>
+      </c>
+      <c r="X11" s="801" t="inlineStr">
+        <is>
+          <t>#ff786f</t>
+        </is>
+      </c>
+      <c r="Y11" s="802" t="inlineStr">
+        <is>
+          <t>#5c6c80</t>
+        </is>
+      </c>
+      <c r="Z11" s="803" t="inlineStr">
+        <is>
+          <t>#c8262a</t>
         </is>
       </c>
       <c r="AA11" t="inlineStr">
         <is>
           <t>/rBkptJyAMqCfoMwUGQfCpubroec.jpg</t>
+        </is>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
All Quiet on the Western Front: point colour from the soldier's face
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q8auJtZCZpXRhnY2W8Jqqg
</commit_message>
<xml_diff>
--- a/data/films.xlsx
+++ b/data/films.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="262">
+  <fonts count="264">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -1068,8 +1068,16 @@
       <b val="1"/>
       <color rgb="00ff786f"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00d57a61"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00cf9787"/>
+    </font>
   </fonts>
-  <fills count="531">
+  <fills count="532">
     <fill>
       <patternFill/>
     </fill>
@@ -3717,6 +3725,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00283546"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00a67162"/>
       </patternFill>
     </fill>
   </fills>
@@ -3732,7 +3745,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="804">
+  <cellXfs count="807">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -4543,6 +4556,9 @@
     <xf numFmtId="0" fontId="261" fillId="530" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="56" fillId="528" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="56" fillId="529" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="262" fillId="390" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="531" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="263" fillId="390" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -6739,9 +6755,9 @@
           <t>#0d2746</t>
         </is>
       </c>
-      <c r="X13" s="599" t="inlineStr">
-        <is>
-          <t>#4399d3</t>
+      <c r="X13" s="806" t="inlineStr">
+        <is>
+          <t>#cf9787</t>
         </is>
       </c>
       <c r="Y13" s="600" t="inlineStr">
@@ -6749,14 +6765,19 @@
           <t>#113157</t>
         </is>
       </c>
-      <c r="Z13" s="601" t="inlineStr">
-        <is>
-          <t>#6a8193</t>
+      <c r="Z13" s="805" t="inlineStr">
+        <is>
+          <t>#a67162</t>
         </is>
       </c>
       <c r="AA13" t="inlineStr">
         <is>
           <t>/fGUK8G7xNLocT4w0DiMBjTECfqr.jpg</t>
+        </is>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Society of the Snow sky blue with amber flare; Amélie green with yellow
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q8auJtZCZpXRhnY2W8Jqqg
</commit_message>
<xml_diff>
--- a/data/films.xlsx
+++ b/data/films.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="264">
+  <fonts count="266">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -1076,8 +1076,16 @@
       <b val="1"/>
       <color rgb="00cf9787"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00e3b64f"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00e0c344"/>
+    </font>
   </fonts>
-  <fills count="532">
+  <fills count="540">
     <fill>
       <patternFill/>
     </fill>
@@ -3730,6 +3738,46 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00a67162"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0084a5b2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00d8b976"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00023949"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="006295b8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00023855"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00087335"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00e0c344"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000c3c1c"/>
       </patternFill>
     </fill>
   </fills>
@@ -3745,7 +3793,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="807">
+  <cellXfs count="818">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -4559,6 +4607,17 @@
     <xf numFmtId="0" fontId="262" fillId="390" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="55" fillId="531" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="263" fillId="390" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="534" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="264" fillId="534" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="532" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="533" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="536" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="264" fillId="536" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="535" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="539" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="265" fillId="539" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="537" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="538" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -6882,24 +6941,24 @@
           <t>bold</t>
         </is>
       </c>
-      <c r="W14" s="532" t="inlineStr">
-        <is>
-          <t>#1f282c</t>
-        </is>
-      </c>
-      <c r="X14" s="711" t="inlineStr">
-        <is>
-          <t>#119fc6</t>
-        </is>
-      </c>
-      <c r="Y14" s="712" t="inlineStr">
-        <is>
-          <t>#b7cac1</t>
-        </is>
-      </c>
-      <c r="Z14" s="713" t="inlineStr">
-        <is>
-          <t>#6f909d</t>
+      <c r="W14" s="811" t="inlineStr">
+        <is>
+          <t>#023855</t>
+        </is>
+      </c>
+      <c r="X14" s="812" t="inlineStr">
+        <is>
+          <t>#e3b64f</t>
+        </is>
+      </c>
+      <c r="Y14" s="813" t="inlineStr">
+        <is>
+          <t>#6295b8</t>
+        </is>
+      </c>
+      <c r="Z14" s="810" t="inlineStr">
+        <is>
+          <t>#d8b976</t>
         </is>
       </c>
       <c r="AA14" t="inlineStr">
@@ -7010,24 +7069,29 @@
           <t>hand</t>
         </is>
       </c>
-      <c r="W15" s="512" t="inlineStr">
-        <is>
-          <t>#222823</t>
-        </is>
-      </c>
-      <c r="X15" s="513" t="inlineStr">
-        <is>
-          <t>#2aa858</t>
-        </is>
-      </c>
-      <c r="Y15" s="514" t="inlineStr">
-        <is>
-          <t>#090909</t>
-        </is>
-      </c>
-      <c r="Z15" s="515" t="inlineStr">
-        <is>
-          <t>#049648</t>
+      <c r="W15" s="814" t="inlineStr">
+        <is>
+          <t>#0c3c1c</t>
+        </is>
+      </c>
+      <c r="X15" s="815" t="inlineStr">
+        <is>
+          <t>#e0c344</t>
+        </is>
+      </c>
+      <c r="Y15" s="816" t="inlineStr">
+        <is>
+          <t>#087335</t>
+        </is>
+      </c>
+      <c r="Z15" s="817" t="inlineStr">
+        <is>
+          <t>#e0c344</t>
+        </is>
+      </c>
+      <c r="AC15" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Snowy mountain banner for Society of the Snow
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q8auJtZCZpXRhnY2W8Jqqg
</commit_message>
<xml_diff>
--- a/data/films.xlsx
+++ b/data/films.xlsx
@@ -6933,7 +6933,7 @@
       </c>
       <c r="U14" s="3" t="inlineStr">
         <is>
-          <t>peaks</t>
+          <t>snowpeaks</t>
         </is>
       </c>
       <c r="V14" t="inlineStr">
@@ -11604,7 +11604,7 @@
       <formula1>"O"</formula1>
     </dataValidation>
     <dataValidation sqref="U2:U500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"arcade,sun,waves,bands,rings,split,peaks,arch,rays,grid,dots,trees"</formula1>
+      <formula1>"arcade,snowpeaks,sun,waves,bands,rings,split,peaks,arch,rays,grid,dots,trees"</formula1>
     </dataValidation>
     <dataValidation sqref="V2:V500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"classic,elegant,noir,epic,typewriter,mono,bold,scifi,gothic,western,retro,script,hand,comic,light,neon"</formula1>

</xml_diff>

<commit_message>
Pan's Labyrinth: point colour from the tree bark
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q8auJtZCZpXRhnY2W8Jqqg
</commit_message>
<xml_diff>
--- a/data/films.xlsx
+++ b/data/films.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="266">
+  <fonts count="269">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -1084,8 +1084,20 @@
       <b val="1"/>
       <color rgb="00e0c344"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00b3a47a"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00b4a282"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00c0a170"/>
+    </font>
   </fonts>
-  <fills count="540">
+  <fills count="542">
     <fill>
       <patternFill/>
     </fill>
@@ -3778,6 +3790,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="000c3c1c"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00776e55"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00806f50"/>
       </patternFill>
     </fill>
   </fills>
@@ -3793,7 +3815,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="818">
+  <cellXfs count="823">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -4618,6 +4640,11 @@
     <xf numFmtId="0" fontId="265" fillId="539" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="55" fillId="537" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="55" fillId="538" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="266" fillId="247" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="540" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="267" fillId="247" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="541" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="268" fillId="247" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -7453,9 +7480,9 @@
           <t>#20282c</t>
         </is>
       </c>
-      <c r="X18" s="720" t="inlineStr">
-        <is>
-          <t>#31a2d2</t>
+      <c r="X18" s="822" t="inlineStr">
+        <is>
+          <t>#c0a170</t>
         </is>
       </c>
       <c r="Y18" s="721" t="inlineStr">
@@ -7463,9 +7490,9 @@
           <t>#182a2a</t>
         </is>
       </c>
-      <c r="Z18" s="722" t="inlineStr">
-        <is>
-          <t>#57a0c3</t>
+      <c r="Z18" s="821" t="inlineStr">
+        <is>
+          <t>#806f50</t>
         </is>
       </c>
       <c r="AA18" t="inlineStr">

</xml_diff>

<commit_message>
Society of the Snow: original peaks banner in icy colours (new 배너색 column)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q8auJtZCZpXRhnY2W8Jqqg
</commit_message>
<xml_diff>
--- a/data/films.xlsx
+++ b/data/films.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="269">
+  <fonts count="270">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -1095,6 +1095,10 @@
     <font>
       <b val="1"/>
       <color rgb="00c0a170"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00dbe7ee"/>
     </font>
   </fonts>
   <fills count="542">
@@ -3815,7 +3819,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="823">
+  <cellXfs count="824">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -4645,6 +4649,7 @@
     <xf numFmtId="0" fontId="267" fillId="247" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="56" fillId="541" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="268" fillId="247" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="269" fillId="536" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -5010,7 +5015,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -5118,6 +5123,13 @@
       <c r="A17" t="inlineStr">
         <is>
           <t>13. 색고정: O로 표시한 영화는 'Poster colours'를 다시 실행해도 배경색·포인트색·포스터를 바꾸지 않습니다(직접 지정한 색 보호).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>14. 배너색: 상세 페이지 배너 무늬의 색(#aabbcc). 비우면 포인트색 계열을 씁니다. 포인트색과 배너 색을 따로 정하고 싶을 때 사용합니다.</t>
         </is>
       </c>
     </row>
@@ -5132,7 +5144,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC51"/>
+  <dimension ref="A1:AD51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -5164,6 +5176,7 @@
     <col width="30" customWidth="1" min="27" max="27"/>
     <col width="14" customWidth="1" min="28" max="28"/>
     <col width="8" customWidth="1" min="29" max="29"/>
+    <col width="10" customWidth="1" min="30" max="30"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5312,6 +5325,11 @@
           <t>색고정</t>
         </is>
       </c>
+      <c r="AD1" s="5" t="inlineStr">
+        <is>
+          <t>배너색</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -6960,7 +6978,7 @@
       </c>
       <c r="U14" s="3" t="inlineStr">
         <is>
-          <t>snowpeaks</t>
+          <t>peaks</t>
         </is>
       </c>
       <c r="V14" t="inlineStr">
@@ -6996,6 +7014,11 @@
       <c r="AC14" t="inlineStr">
         <is>
           <t>O</t>
+        </is>
+      </c>
+      <c r="AD14" s="823" t="inlineStr">
+        <is>
+          <t>#dbe7ee</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Shoplifters: sunlight yellow base, leafy green point
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q8auJtZCZpXRhnY2W8Jqqg
</commit_message>
<xml_diff>
--- a/data/films.xlsx
+++ b/data/films.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="270">
+  <fonts count="272">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -1100,8 +1100,16 @@
       <b val="1"/>
       <color rgb="00dbe7ee"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="0063c8a4"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="0087c571"/>
+    </font>
   </fonts>
-  <fills count="542">
+  <fills count="545">
     <fill>
       <patternFill/>
     </fill>
@@ -3804,6 +3812,21 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00806f50"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00d8b77c"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0049695c"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00463103"/>
       </patternFill>
     </fill>
   </fills>
@@ -3819,7 +3842,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="824">
+  <cellXfs count="829">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -4650,6 +4673,11 @@
     <xf numFmtId="0" fontId="56" fillId="541" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="268" fillId="247" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="269" fillId="536" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="544" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="270" fillId="544" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="542" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="543" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="271" fillId="544" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -7626,24 +7654,24 @@
           <t>elegant</t>
         </is>
       </c>
-      <c r="W19" s="723" t="inlineStr">
-        <is>
-          <t>#29261e</t>
-        </is>
-      </c>
-      <c r="X19" s="724" t="inlineStr">
-        <is>
-          <t>#13a2ad</t>
-        </is>
-      </c>
-      <c r="Y19" s="725" t="inlineStr">
-        <is>
-          <t>#2e2b23</t>
-        </is>
-      </c>
-      <c r="Z19" s="726" t="inlineStr">
-        <is>
-          <t>#3c5b5e</t>
+      <c r="W19" s="824" t="inlineStr">
+        <is>
+          <t>#463103</t>
+        </is>
+      </c>
+      <c r="X19" s="828" t="inlineStr">
+        <is>
+          <t>#87c571</t>
+        </is>
+      </c>
+      <c r="Y19" s="826" t="inlineStr">
+        <is>
+          <t>#d8b77c</t>
+        </is>
+      </c>
+      <c r="Z19" s="827" t="inlineStr">
+        <is>
+          <t>#49695c</t>
         </is>
       </c>
       <c r="AA19" t="inlineStr">

</xml_diff>

<commit_message>
Chungking Express mint with yellow; Léon dark crimson with yellow
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q8auJtZCZpXRhnY2W8Jqqg
</commit_message>
<xml_diff>
--- a/data/films.xlsx
+++ b/data/films.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="272">
+  <fonts count="278">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -1108,8 +1108,32 @@
       <b val="1"/>
       <color rgb="0087c571"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00ceb236"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00ddc123"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00d3b708"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00edd13d"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="008fd3c1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00fdae20"/>
+    </font>
   </fonts>
-  <fills count="545">
+  <fills count="553">
     <fill>
       <patternFill/>
     </fill>
@@ -3827,6 +3851,46 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00463103"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0073a18f"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00c9b14f"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00023b2c"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00023a36"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00f60d0d"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00f4a609"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00581c16"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004c0b13"/>
       </patternFill>
     </fill>
   </fills>
@@ -3842,7 +3906,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="829">
+  <cellXfs count="844">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -4678,6 +4742,21 @@
     <xf numFmtId="0" fontId="55" fillId="542" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="55" fillId="543" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="271" fillId="544" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="547" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="272" fillId="547" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="545" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="546" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="273" fillId="547" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="548" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="274" fillId="548" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="275" fillId="548" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="276" fillId="548" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="551" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="277" fillId="551" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="549" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="550" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="552" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="277" fillId="552" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -11288,24 +11367,24 @@
           <t>bold</t>
         </is>
       </c>
-      <c r="W48" s="416" t="inlineStr">
-        <is>
-          <t>#2d2422</t>
-        </is>
-      </c>
-      <c r="X48" s="774" t="inlineStr">
-        <is>
-          <t>#f06753</t>
-        </is>
-      </c>
-      <c r="Y48" s="775" t="inlineStr">
-        <is>
-          <t>#010102</t>
-        </is>
-      </c>
-      <c r="Z48" s="776" t="inlineStr">
-        <is>
-          <t>#b22c1c</t>
+      <c r="W48" s="842" t="inlineStr">
+        <is>
+          <t>#4c0b13</t>
+        </is>
+      </c>
+      <c r="X48" s="843" t="inlineStr">
+        <is>
+          <t>#fdae20</t>
+        </is>
+      </c>
+      <c r="Y48" s="840" t="inlineStr">
+        <is>
+          <t>#f60d0d</t>
+        </is>
+      </c>
+      <c r="Z48" s="841" t="inlineStr">
+        <is>
+          <t>#f4a609</t>
         </is>
       </c>
       <c r="AA48" t="inlineStr">
@@ -11416,24 +11495,34 @@
           <t>neon</t>
         </is>
       </c>
-      <c r="W49" s="573" t="inlineStr">
-        <is>
-          <t>#371f1c</t>
-        </is>
-      </c>
-      <c r="X49" s="574" t="inlineStr">
-        <is>
-          <t>#cbaa3f</t>
-        </is>
-      </c>
-      <c r="Y49" s="296" t="inlineStr">
-        <is>
-          <t>#301512</t>
-        </is>
-      </c>
-      <c r="Z49" s="297" t="inlineStr">
-        <is>
-          <t>#cbaa3f</t>
+      <c r="W49" s="834" t="inlineStr">
+        <is>
+          <t>#023a36</t>
+        </is>
+      </c>
+      <c r="X49" s="836" t="inlineStr">
+        <is>
+          <t>#edd13d</t>
+        </is>
+      </c>
+      <c r="Y49" s="831" t="inlineStr">
+        <is>
+          <t>#73a18f</t>
+        </is>
+      </c>
+      <c r="Z49" s="832" t="inlineStr">
+        <is>
+          <t>#c9b14f</t>
+        </is>
+      </c>
+      <c r="AC49" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="AD49" s="837" t="inlineStr">
+        <is>
+          <t>#8fd3c1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Your Name.: twilight orange point
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q8auJtZCZpXRhnY2W8Jqqg
</commit_message>
<xml_diff>
--- a/data/films.xlsx
+++ b/data/films.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="278">
+  <fonts count="279">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -1131,6 +1131,10 @@
     <font>
       <b val="1"/>
       <color rgb="00fdae20"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00fe8e41"/>
     </font>
   </fonts>
   <fills count="553">
@@ -3906,7 +3910,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="844">
+  <cellXfs count="845">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -4757,6 +4761,7 @@
     <xf numFmtId="0" fontId="55" fillId="550" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="552" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="277" fillId="552" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="278" fillId="368" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -10378,9 +10383,9 @@
           <t>#042847</t>
         </is>
       </c>
-      <c r="X40" s="560" t="inlineStr">
-        <is>
-          <t>#6492df</t>
+      <c r="X40" s="844" t="inlineStr">
+        <is>
+          <t>#fe8e41</t>
         </is>
       </c>
       <c r="Y40" s="261" t="inlineStr">
@@ -10391,6 +10396,11 @@
       <c r="Z40" s="262" t="inlineStr">
         <is>
           <t>#325da6</t>
+        </is>
+      </c>
+      <c r="AC40" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Placeholders drawn in each film's banner colours; Mononoke green forest; softly rounded popups
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q8auJtZCZpXRhnY2W8Jqqg
</commit_message>
<xml_diff>
--- a/data/films.xlsx
+++ b/data/films.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="280">
+  <fonts count="281">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -1139,6 +1139,10 @@
     <font>
       <b val="1"/>
       <color rgb="00ff61c5"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="007fb069"/>
     </font>
   </fonts>
   <fills count="553">
@@ -3914,7 +3918,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="846">
+  <cellXfs count="847">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -4767,6 +4771,7 @@
     <xf numFmtId="0" fontId="277" fillId="552" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="278" fillId="368" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="279" fillId="425" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="280" fillId="283" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -9519,6 +9524,11 @@
           <t>#b51b11</t>
         </is>
       </c>
+      <c r="AD33" s="846" t="inlineStr">
+        <is>
+          <t>#7fb069</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Inside Out: yellow point
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q8auJtZCZpXRhnY2W8Jqqg
</commit_message>
<xml_diff>
--- a/data/films.xlsx
+++ b/data/films.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="281">
+  <fonts count="282">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -1143,6 +1143,10 @@
     <font>
       <b val="1"/>
       <color rgb="007fb069"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00f2d935"/>
     </font>
   </fonts>
   <fills count="553">
@@ -3918,7 +3922,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="847">
+  <cellXfs count="848">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -4772,6 +4776,7 @@
     <xf numFmtId="0" fontId="278" fillId="368" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="279" fillId="425" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="280" fillId="283" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="281" fillId="514" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -10147,9 +10152,9 @@
           <t>#192348</t>
         </is>
       </c>
-      <c r="X38" s="783" t="inlineStr">
-        <is>
-          <t>#e6698a</t>
+      <c r="X38" s="847" t="inlineStr">
+        <is>
+          <t>#f2d935</t>
         </is>
       </c>
       <c r="Y38" s="784" t="inlineStr">

</xml_diff>

<commit_message>
Comic-city banner for Spider-Man: halftone, burst lines, skyline
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q8auJtZCZpXRhnY2W8Jqqg
</commit_message>
<xml_diff>
--- a/data/films.xlsx
+++ b/data/films.xlsx
@@ -9873,7 +9873,7 @@
       </c>
       <c r="U36" s="3" t="inlineStr">
         <is>
-          <t>dots</t>
+          <t>comic</t>
         </is>
       </c>
       <c r="V36" t="inlineStr">
@@ -11801,7 +11801,7 @@
       <formula1>"O"</formula1>
     </dataValidation>
     <dataValidation sqref="U2:U500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"arcade,snowpeaks,sun,waves,bands,rings,split,peaks,arch,rays,grid,dots,trees"</formula1>
+      <formula1>"comic,arcade,snowpeaks,sun,waves,bands,rings,split,peaks,arch,rays,grid,dots,trees"</formula1>
     </dataValidation>
     <dataValidation sqref="V2:V500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"classic,elegant,noir,epic,typewriter,mono,bold,scifi,gothic,western,retro,script,hand,comic,light,neon"</formula1>

</xml_diff>

<commit_message>
The Godfather: near-black base, gold point
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q8auJtZCZpXRhnY2W8Jqqg
</commit_message>
<xml_diff>
--- a/data/films.xlsx
+++ b/data/films.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="282">
+  <fonts count="283">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -1148,8 +1148,12 @@
       <b val="1"/>
       <color rgb="00f2d935"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00deb866"/>
+    </font>
   </fonts>
-  <fills count="553">
+  <fills count="554">
     <fill>
       <patternFill/>
     </fill>
@@ -3907,6 +3911,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="004c0b13"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00110f0d"/>
       </patternFill>
     </fill>
   </fills>
@@ -3922,7 +3931,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="848">
+  <cellXfs count="850">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -4777,6 +4786,8 @@
     <xf numFmtId="0" fontId="279" fillId="425" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="280" fillId="283" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="281" fillId="514" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="553" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="282" fillId="553" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -10649,14 +10660,14 @@
           <t>noir</t>
         </is>
       </c>
-      <c r="W42" s="335" t="inlineStr">
-        <is>
-          <t>#2c2520</t>
-        </is>
-      </c>
-      <c r="X42" s="562" t="inlineStr">
-        <is>
-          <t>#cb8043</t>
+      <c r="W42" s="848" t="inlineStr">
+        <is>
+          <t>#110f0d</t>
+        </is>
+      </c>
+      <c r="X42" s="849" t="inlineStr">
+        <is>
+          <t>#deb866</t>
         </is>
       </c>
       <c r="Y42" s="269" t="inlineStr">
@@ -10667,6 +10678,11 @@
       <c r="Z42" s="270" t="inlineStr">
         <is>
           <t>#b87238</t>
+        </is>
+      </c>
+      <c r="AC42" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Per-film banner scenes for 47 films, motif tweaks
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q8auJtZCZpXRhnY2W8Jqqg
</commit_message>
<xml_diff>
--- a/data/films.xlsx
+++ b/data/films.xlsx
@@ -7761,7 +7761,7 @@
       </c>
       <c r="U19" s="3" t="inlineStr">
         <is>
-          <t>split</t>
+          <t>waves</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
@@ -9766,7 +9766,7 @@
       </c>
       <c r="U35" s="3" t="inlineStr">
         <is>
-          <t>dots</t>
+          <t>snowpeaks</t>
         </is>
       </c>
       <c r="V35" t="inlineStr">
@@ -10662,7 +10662,7 @@
       </c>
       <c r="U42" s="3" t="inlineStr">
         <is>
-          <t>rays</t>
+          <t>split</t>
         </is>
       </c>
       <c r="V42" t="inlineStr">
@@ -10785,7 +10785,7 @@
       </c>
       <c r="U43" s="3" t="inlineStr">
         <is>
-          <t>rays</t>
+          <t>grid</t>
         </is>
       </c>
       <c r="V43" t="inlineStr">
@@ -11543,7 +11543,7 @@
       </c>
       <c r="U49" s="3" t="inlineStr">
         <is>
-          <t>bands</t>
+          <t>dots</t>
         </is>
       </c>
       <c r="V49" t="inlineStr">
@@ -11789,7 +11789,7 @@
       </c>
       <c r="U51" s="3" t="inlineStr">
         <is>
-          <t>split</t>
+          <t>bands</t>
         </is>
       </c>
       <c r="V51" t="inlineStr">

</xml_diff>

<commit_message>
The Dark Knight: red-orange point
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q8auJtZCZpXRhnY2W8Jqqg
</commit_message>
<xml_diff>
--- a/data/films.xlsx
+++ b/data/films.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="284">
+  <fonts count="285">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -1155,6 +1155,10 @@
     <font>
       <b val="1"/>
       <color rgb="00fe9d39"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00fe7644"/>
     </font>
   </fonts>
   <fills count="554">
@@ -3935,7 +3939,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="851">
+  <cellXfs count="852">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -4793,6 +4797,7 @@
     <xf numFmtId="0" fontId="3" fillId="553" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="282" fillId="553" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="283" fillId="425" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="284" fillId="247" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -8659,9 +8664,9 @@
           <t>#20282c</t>
         </is>
       </c>
-      <c r="X26" s="740" t="inlineStr">
-        <is>
-          <t>#329cce</t>
+      <c r="X26" s="851" t="inlineStr">
+        <is>
+          <t>#fe7644</t>
         </is>
       </c>
       <c r="Y26" s="205" t="inlineStr">

</xml_diff>

<commit_message>
Shoplifters: green background, yellow point
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q8auJtZCZpXRhnY2W8Jqqg
</commit_message>
<xml_diff>
--- a/data/films.xlsx
+++ b/data/films.xlsx
@@ -7776,12 +7776,12 @@
       </c>
       <c r="W19" s="824" t="inlineStr">
         <is>
-          <t>#463103</t>
+          <t>#254a1f</t>
         </is>
       </c>
       <c r="X19" s="828" t="inlineStr">
         <is>
-          <t>#87c571</t>
+          <t>#f2d64b</t>
         </is>
       </c>
       <c r="Y19" s="826" t="inlineStr">

</xml_diff>

<commit_message>
Perfect Days: green background
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q8auJtZCZpXRhnY2W8Jqqg
</commit_message>
<xml_diff>
--- a/data/films.xlsx
+++ b/data/films.xlsx
@@ -7904,7 +7904,7 @@
       </c>
       <c r="W20" s="616" t="inlineStr">
         <is>
-          <t>#312319</t>
+          <t>#1f4a2a</t>
         </is>
       </c>
       <c r="X20" s="617" t="inlineStr">
@@ -7925,6 +7925,11 @@
       <c r="AA20" t="inlineStr">
         <is>
           <t>/4UyKNimG5VHTcGjOH3z5kJFndLM.jpg</t>
+        </is>
+      </c>
+      <c r="AC20" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync data with main; soften Shoplifters horizon less aggressively
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q8auJtZCZpXRhnY2W8Jqqg
</commit_message>
<xml_diff>
--- a/data/films.xlsx
+++ b/data/films.xlsx
@@ -7776,7 +7776,7 @@
       </c>
       <c r="W19" s="824" t="inlineStr">
         <is>
-          <t>#3f8f2e</t>
+          <t>#254a1f</t>
         </is>
       </c>
       <c r="X19" s="828" t="inlineStr">
@@ -7909,7 +7909,7 @@
       </c>
       <c r="X20" s="617" t="inlineStr">
         <is>
-          <t>#808cdd</t>
+          <t>#c3c9ff</t>
         </is>
       </c>
       <c r="Y20" s="618" t="inlineStr">

</xml_diff>

<commit_message>
Life Is Beautiful: navy background, near-white sky-blue point
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q8auJtZCZpXRhnY2W8Jqqg
</commit_message>
<xml_diff>
--- a/data/films.xlsx
+++ b/data/films.xlsx
@@ -11051,12 +11051,12 @@
       </c>
       <c r="W45" s="785" t="inlineStr">
         <is>
-          <t>#21243e</t>
+          <t>#14224d</t>
         </is>
       </c>
       <c r="X45" s="786" t="inlineStr">
         <is>
-          <t>#cb7f44</t>
+          <t>#dff1ff</t>
         </is>
       </c>
       <c r="Y45" s="787" t="inlineStr">

</xml_diff>

<commit_message>
Shoplifters: teal-leaning green; Perfect Days: green with brown tint
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q8auJtZCZpXRhnY2W8Jqqg
</commit_message>
<xml_diff>
--- a/data/films.xlsx
+++ b/data/films.xlsx
@@ -7776,7 +7776,7 @@
       </c>
       <c r="W19" s="824" t="inlineStr">
         <is>
-          <t>#254a1f</t>
+          <t>#1f4d45</t>
         </is>
       </c>
       <c r="X19" s="828" t="inlineStr">
@@ -7904,7 +7904,7 @@
       </c>
       <c r="W20" s="616" t="inlineStr">
         <is>
-          <t>#1f4a2a</t>
+          <t>#3b4a26</t>
         </is>
       </c>
       <c r="X20" s="617" t="inlineStr">

</xml_diff>